<commit_message>
feat(voice): façade unifiée BaouleVoiceEngine — baoule-engine.ts (B5-050)
- façade PURE sur B1→B4 : getBaouleEngineStatus/isBaouleEngineReady (sondes),
  initializeBaouleEngine (STT natif bci, jamais de téléchargement, état exact),
  createBaouleTranscriptionSession (STT offline, erreur explicite hors natif),
  translateBaouleToFrench/prepareBaouleParserInput (garde B2-022),
  speakBaoule (ne lève jamais), installBaouleTranslator/Voice (opt-in)
- BaouleEngineError (7 codes) + describeBaouleEngineError
- chaque maillon reste dans son module d'origine (source de vérité unique)
- tests contrat 16 cas → suite 598/598 · tsc 0 · lint 0 · build prod OK
- registre : B5-050 → VALIDATION 90 % (TASKS.xlsx + miroir + CHANGELOG +
  AGENT1_STATUS + HANDOFF n°7)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -2785,7 +2785,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Créer src/lib/voice/baoule-engine.ts : initialize/isReady/transcribe/speak + codes d'erreur dédiés ; encapsule B1→B4.</t>
+          <t>Façade B1→B4 livrée : getBaouleEngineStatus/isBaouleEngineReady (sonde sans effet de bord), initializeBaouleEngine (charge le STT natif bci, NE TÉLÉCHARGE JAMAIS, état exact des maillons manquants), createBaouleTranscriptionSession (STT offline, session inerte explicite hors natif), translateBaouleToFrench + prepareBaouleParserInput (garde B2-022, erreurs mappées), speakBaoule (ne lève jamais, repli explicite), installBaouleTranslator/installBaouleVoice (opt-in). BaouleEngineError 7 codes + describeBaouleEngineError.</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -2793,13 +2793,13 @@
           <t>AGENT 1</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+      <c r="H29" s="11" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
         </is>
       </c>
       <c r="I29" s="6" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
@@ -2813,12 +2813,12 @@
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>src/lib/voice/baoule-engine.ts (à créer)</t>
+          <t>src/lib/voice/baoule-engine.ts (nouveau) — façade pure, chaque maillon reste dans son module d'origine</t>
         </is>
       </c>
       <c r="M29" s="4" t="inlineStr">
         <is>
-          <t>Tests de contrat</t>
+          <t>16 tests contrat · 598/598 · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N29" s="4" t="inlineStr">
@@ -2845,7 +2845,7 @@
       <c r="S29" s="4" t="inlineStr"/>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>Pattern voice-service.ts ; garde-fous mission préservés</t>
+          <t>Branchement stt-factory/modales = B5-051 ; smoke APK = B5-052</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(voice): brancher la façade BaouleVoiceEngine — stt-factory + modales (B5-051)
- stt-factory : route bci → createBaouleTranscriptionSession (délégation
  VoiceService, comportement identique) ; route fr inchangée
- voice-modal + prod-voice-modal : migration façade (prepareBaouleParserInput /
  speakBaoule / describeBaouleEngineError) — entrée UNIQUE de la chaîne baoulé
- baoule-engine : ré-export fetchJsonWithTimeout + CONVERSATION_NETWORK_TIMEOUT_MS
- stt-routing.test.ts : mock registerPlugin complété (chaîne façade → native-tts)
- non-régression fr : 32 tata-tts + 21 stt-routing/factory verts · 598/598 ·
  tsc 0 · lint 0 · build prod OK
- registre : B5-051 → VALIDATION 90 % (TASKS.xlsx + miroir + CHANGELOG +
  AGENT1_STATUS + HANDOFF n°8)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -2872,7 +2872,7 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>Brancher stt-factory (bci → engine) + voice-modal + prod-voice-modal ; non-régression française.</t>
+          <t>Branchement livré : stt-factory route le bci via createBaouleTranscriptionSession (façade — délégation VoiceService, comportement identique) ; les 2 modales migrent vers la façade (prepareBaouleParserInput / speakBaoule / describeBaouleEngineError / fetchJsonWithTimeout ré-exporté) — BaouleVoiceEngine est l'entrée UNIQUE de la chaîne baoulé côté UI. Non-régression fr : route fr de stt-factory inchangée, 32 tests tata-tts verts.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -2880,13 +2880,13 @@
           <t>AGENT 1</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
         </is>
       </c>
       <c r="I30" s="9" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
@@ -2900,12 +2900,12 @@
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
-          <t>stt-factory.ts, voice-modal.tsx, prod-voice-modal.tsx</t>
+          <t>stt-factory.ts, voice-modal.tsx, prod-voice-modal.tsx, baoule-engine.ts (ré-export réseau)</t>
         </is>
       </c>
       <c r="M30" s="7" t="inlineStr">
         <is>
-          <t>stt-routing étendu</t>
+          <t>598/598 (38 fichiers) · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N30" s="7" t="inlineStr">
@@ -2930,7 +2930,11 @@
         </is>
       </c>
       <c r="S30" s="7" t="inlineStr"/>
-      <c r="T30" s="7" t="inlineStr"/>
+      <c r="T30" s="7" t="inlineStr">
+        <is>
+          <t>Smoke APK = B5-052 (AGENT 2) ; mock registerPlugin ajouté à stt-routing (chaîne façade → native-tts)</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="B31" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore(cleanup): supprimer le code mort vérifié (NORM-302)
- src/lib/supabase/browser.ts, ident-top-bar.tsx, db/custom.db,
  examples/websocket/ : 0 importeur confirmé partout
- dep z-ai-web-dev-sdk retirée (package.json + bun.lock synchronisés)
- 598/598 · tsc 0 · lint 0 · build prod OK · CSP intacte
- registre : NORM-302 → TERMINÉ (TASKS.xlsx + miroir + CHANGELOG +
  AGENT1_STATUS)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -3224,7 +3224,7 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>supabase/browser.ts, ident-top-bar.tsx, db/custom.db (vestige Prisma), examples/websocket, dep z-ai-web-dev-sdk.</t>
+          <t>Supprimé et vérifié (0 importeur partout) : src/lib/supabase/browser.ts, src/components/identificateur/ident-top-bar.tsx, db/custom.db (vestige Prisma), examples/websocket/, dépendance z-ai-web-dev-sdk (package.json + bun.lock synchronisés, 1 paquet retiré). Référence z-ai restante dans tests/python-runtime-container.sh = nom d'image Docker, sans rapport.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -3232,13 +3232,13 @@
           <t>AGENT 1</t>
         </is>
       </c>
-      <c r="H34" s="7" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I34" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="M34" s="7" t="inlineStr">
         <is>
-          <t>build + tests + lint</t>
+          <t>598/598 · tsc 0 · lint 0 · build prod OK · CSP intacte</t>
         </is>
       </c>
       <c r="N34" s="7" t="inlineStr">
@@ -3284,7 +3284,7 @@
       <c r="S34" s="7" t="inlineStr"/>
       <c r="T34" s="7" t="inlineStr">
         <is>
-          <t>Zéro impact fonctionnel attendu</t>
+          <t>Zéro impact fonctionnel confirmé ; lockfiles unifiés = NORM-303 (backlog)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: aligner AGENTS.md sur la réalité du dépôt (DOC-306)
- 10 stores nommés (gemma-model, network, voice-language manquants)
- pipeline voix réel : STT natif (sherpa FR + Omnilingual bci) via
  stt-factory, TTS tata-tts + Piper/Kokoro opt-in + voix MMS bci,
  NLLB + façade BaouleVoiceEngine, Web Speech = repli web fr
- arborescence voice/ détaillée
- registre : DOC-306 → TERMINÉ (TASKS.xlsx + miroir + CHANGELOG +
  AGENT1_STATUS)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -3548,7 +3548,7 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>AGENTS.md obsolète : « 7 stores » (réel 10), pipeline voix décrit « Web Speech » (réel 3 STT + 4 TTS), Tasks 31-40 absentes.</t>
+          <t>AGENTS.md aligné : « 10 stores » (app, backoffice, caisse, gemma-model, identificateur, network, notifications, producteur, stock, voice-language) ; pipeline voix réel (STT natif VoiceService + Omnilingual bci via stt-factory ; TTS tata-tts + Piper/Kokoro opt-in + voix MMS bci pilote ; NLLB + façade BaouleVoiceEngine ; Web Speech = repli web fr uniquement) ; arborescence voice/ détaillée.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -3556,13 +3556,13 @@
           <t>AGENT 1</t>
         </is>
       </c>
-      <c r="H38" s="7" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I38" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="M38" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Doc seule — zéro impact runtime (baseline 598/598 inchangée)</t>
         </is>
       </c>
       <c r="N38" s="7" t="inlineStr">

</xml_diff>

<commit_message>
test(e2e): chaîne conversation baoulé de bout en bout (B4-042, AGENT 2)
- baoule-chain-e2e.test.ts : 5 scénarios — tour complet STT bci → trad fr
  → intent vente → confirmation ɛhɛ/ao → NLLB fra→bci → TTS bci ;
  garde de bout en bout (parseIntent jamais atteint si traducteur absent) ;
  repli français hors MMS ; non-régression fr dédiée
- maillons métier RÉELS (baoule-engine, conversation, localIntent,
  confirmations) — mocks aux seules frontières externes
- verdicts AGENT 2 : B4-042 TERMINÉ · B5-052 BLOQUÉ (appareil requis) ·
  6 tâches VALIDATION 90 % confirmées
- suite 603/603 (39 fichiers) · tsc 0 · lint 0 · build prod OK
- registre : TASKS.xlsx + miroir + CHANGELOG + AGENT2_STATUS
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -2698,7 +2698,7 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>Dictée bci → vente confirmée → TTS bci ; non-régression des 33 suites.</t>
+          <t>baoule-chain-e2e.test.ts (AGENT 2) : 5 scénarios — tour complet STT bci → trad fr → intent vente (2000 F, tomate) → confirm ɛhɛ/ao → NLLB fra→bci → tataSpeak texte brut bci ; garde de bout en bout (parseIntent jamais atteint si traducteur absent) ; repli français hors MMS ; non-régression fr dédiée.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -2706,13 +2706,13 @@
           <t>AGENT 2</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I28" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
@@ -2726,12 +2726,12 @@
       </c>
       <c r="L28" s="7" t="inlineStr">
         <is>
-          <t>src/lib/voice/__tests__/</t>
+          <t>src/lib/voice/__tests__/baoule-chain-e2e.test.ts</t>
         </is>
       </c>
       <c r="M28" s="7" t="inlineStr">
         <is>
-          <t>Suite chaîne bci</t>
+          <t>5/5 · suite 603/603 · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N28" s="7" t="inlineStr">
@@ -2758,7 +2758,7 @@
       <c r="S28" s="7" t="inlineStr"/>
       <c r="T28" s="7" t="inlineStr">
         <is>
-          <t>TEST_PLAN §3-B4</t>
+          <t>TEST_PLAN §3-B4 ; validation device regroupée B1-010/B3-032/B5-052</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Tests de contrat + routing + smoke APK (assembleDebug + conversation bci de bout en bout sur appareil).</t>
+          <t>Volet contrat COUVERT (baoule-engine.test.ts 16 cas + baoule-chain-e2e.test.ts 5 scénarios, validés AGENT 2). Smoke APK (assembleDebug + conversation bci de bout en bout sur téléphone) : APPAREIL REQUIS — sessions terrain regroupées avec B1-010/B2-021/B3-031/B3-032.</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -2967,13 +2967,13 @@
           <t>AGENT 2</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>BLOQUÉ</t>
         </is>
       </c>
       <c r="I31" s="6" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>Smoke APK</t>
+          <t>assembleDebug + conversation device</t>
         </is>
       </c>
       <c r="N31" s="4" t="inlineStr">
@@ -3019,7 +3019,7 @@
       <c r="S31" s="4" t="inlineStr"/>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>TEST_PLAN §3-B5</t>
+          <t>TEST_PLAN §3-B5 ; smartphone Tecno/Infinix requis</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
audit(vocal): vente rapide — 2 P0 (STT hors factory → spinner infini APK ; montant dicté écrasé par priceUnit) + 4 P1 + 4 P2, plan VOCAL-602..605 (VOCAL-601)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -123,7 +123,6 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,13 +488,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:T44"/>
+  <dimension ref="A2:T49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
@@ -3615,45 +3614,45 @@
     <row r="39" ht="22" customHeight="1">
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>INF-401</t>
+          <t>VOCAL-601</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Audit vocal</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Déploiement prod + APK</t>
+          <t>Audit vocal vente rapide</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Vercel puis APK autonome</t>
+          <t>Constater pourquoi « ça casse » + plan</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
+          <t>Audit statique complet du parcours vocal VenteRapideModal (rapport .ai/AUDIT_VOCAL_VENTE_RAPIDE.md) : 2 P0 — STT Web Speech brut hors factory (spinner infini « J'écoute... » sur APK, no-op silencieux stt.ts:92) et montant dicté écrasé par le prix catalogue (vente « tomates 2000 » enregistrée au prix du stock) ; 4 P1 — race wake-word à l'ouverture, fetch sans timeout + stock décrémenté avant verdict, watchdog d'écoute absent, sessions STT dupliquées ; 4 P2 — intents non métier, confirmation trop ferme, synced ignoré, hygiène. Preuves fichier:ligne + scénarios chiffrés + critères d'acceptation.</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>ORCHESTRATEUR</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I39" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
@@ -3663,12 +3662,12 @@
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
+          <t>.ai/AUDIT_VOCAL_VENTE_RAPIDE.md</t>
         </is>
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>Smoke APK</t>
+          <t>Audit statique — zéro impact runtime (baseline 603/603 inchangée)</t>
         </is>
       </c>
       <c r="N39" s="4" t="inlineStr">
@@ -3684,55 +3683,55 @@
       </c>
       <c r="Q39" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="R39" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="S39" s="4" t="inlineStr"/>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+          <t>Corrections = VOCAL-602/603/604/605 ; confirmation smoke device du P0-1 (rejoint B1-010/B5-052)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>SEC-402</t>
+          <t>VOCAL-602</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Audit vocal</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>PAT GitHub exposé</t>
+          <t>Factory STT dans la vente rapide</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>Révocation</t>
+          <t>Brancher la modale sur la chaîne multi-moteurs</t>
         </is>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+          <t>Porte canAttemptSTT() au lieu de isAnySTTAvailable() ; session hybride — web : createSingleShotSTT synchrone (préserver l'activation utilisateur documentée), natif : createSmartSingleShotSTT → VoiceService/Sherpa ; watchdog d'écoute 12-15 s avec erreur explicite + repli clavier ; abort systématique de la session précédente + compteur de génération (fin des fuites de micro).</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>USER</t>
-        </is>
-      </c>
-      <c r="H40" s="13" t="inlineStr">
-        <is>
-          <t>BLOQUÉ</t>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
         </is>
       </c>
       <c r="I40" s="9" t="n">
@@ -3745,17 +3744,17 @@
       </c>
       <c r="K40" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VOCAL-601</t>
         </is>
       </c>
       <c r="L40" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>vente-rapide-modal.tsx, stt-factory.ts (helper partagé)</t>
         </is>
       </c>
       <c r="M40" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Tests machine à états + choix moteur</t>
         </is>
       </c>
       <c r="N40" s="7" t="inlineStr">
@@ -3771,32 +3770,467 @@
       </c>
       <c r="Q40" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="R40" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="S40" s="7" t="inlineStr"/>
       <c r="T40" s="7" t="inlineStr">
         <is>
+          <t>Corrige le spinner infini constaté sur APK ; donne le routage Baoulé gratuitement</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>VOCAL-603</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Audit vocal</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Montant dicté = vérité</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Fin de l'override priceUnit + format « X à Y »</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>unitPrice = round(amount/qty) calculé depuis le montant DICTÉ — le priceUnit du stock n'écrase plus jamais la parole du marchand ; « X à Y » → amount = qty × prix unitaire (extractAmount/parseIntent) ; annonce du montant réellement enregistré ; signaler l'écart éventuel avec le prix catalogue au lieu de l'écraser en silence.</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>VOCAL-601</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>vente-rapide-modal.tsx, localIntent.ts</t>
+        </is>
+      </c>
+      <c r="M41" s="4" t="inlineStr">
+        <is>
+          <t>4 scénarios chiffrés de l'audit §P0-2 en tests unitaires</t>
+        </is>
+      </c>
+      <c r="N41" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr"/>
+      <c r="P41" s="4" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q41" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R41" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S41" s="4" t="inlineStr"/>
+      <c r="T41" s="4" t="inlineStr">
+        <is>
+          <t>Impact métier direct : caisse/ventes/objectifs faussés silencieusement</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>VOCAL-604</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Audit vocal</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Race wake-word + réseau/stock</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>Durcir l'arène micro et la persistance</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>resumeWakeWord seulement à la fermeture effective de la modale + pauseWakeWord annule un start en cours (plus de listener de fond pendant la vente rapide) ; fetchJsonWithTimeout (10 s) dans completeQuickSale — plus de « processing » figé ; décrément stock après verdict (succès réseau OU file offline confirmée) ; result.synced annoncé (« sera synchronisée »).</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I42" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>VOCAL-601</t>
+        </is>
+      </c>
+      <c r="L42" s="7" t="inlineStr">
+        <is>
+          <t>vente-rapide-modal.tsx, wake-word.ts, quick-sale.ts</t>
+        </is>
+      </c>
+      <c r="M42" s="7" t="inlineStr">
+        <is>
+          <t>Test : fetch suspendu → erreur à 10 s + file offline</t>
+        </is>
+      </c>
+      <c r="N42" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O42" s="7" t="inlineStr"/>
+      <c r="P42" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q42" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R42" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S42" s="7" t="inlineStr"/>
+      <c r="T42" s="7" t="inlineStr">
+        <is>
+          <t>fetchJsonWithTimeout déjà disponible (B4-041)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>VOCAL-605</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Audit vocal</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Intents non métier + hygiène</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Parcours oui/stop/navigation/consultation</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>« oui » au prompt = nouvelle écoute (fini l'erreur texte vide) ; « stop/annule » ferme poliment la modale ; navigation = fermer puis naviguer (ou message explicite) ; consultation = total réel du jour (caisse-store) ; confirmation : clavier oui/non sur erreur micro, enchaîner une nouvelle vente si réponse ni oui ni non ; retrait code mort (pendingConfirmRef, state error, AMOUNT_PATTERNS) ; typos « Daccord » → « D'accord » ; survente signalée.</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>VOCAL-602</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>vente-rapide-modal.tsx, localIntent.ts</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t>Parcours oui/stop/mes ventes/combien testés</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr"/>
+      <c r="P43" s="4" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q43" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R43" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S43" s="4" t="inlineStr"/>
+      <c r="T43" s="4" t="inlineStr">
+        <is>
+          <t>Barge-in + prompts bci arbitrés séparément</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>INF-401</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Déploiement prod + APK</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>Vercel puis APK autonome</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>ORCHESTRATEUR</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I44" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L44" s="7" t="inlineStr">
+        <is>
+          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
+        </is>
+      </c>
+      <c r="M44" s="7" t="inlineStr">
+        <is>
+          <t>Smoke APK</t>
+        </is>
+      </c>
+      <c r="N44" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O44" s="7" t="inlineStr"/>
+      <c r="P44" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q44" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="R44" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="S44" s="7" t="inlineStr"/>
+      <c r="T44" s="7" t="inlineStr">
+        <is>
+          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>SEC-402</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>PAT GitHub exposé</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Révocation</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="H45" s="10" t="inlineStr">
+        <is>
+          <t>BLOQUÉ</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N45" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr"/>
+      <c r="P45" s="4" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q45" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="R45" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="S45" s="4" t="inlineStr"/>
+      <c r="T45" s="4" t="inlineStr">
+        <is>
           <t>Action utilisateur requise — P0 absolu</t>
         </is>
       </c>
     </row>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43">
-      <c r="B43" s="2" t="inlineStr">
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="2" t="inlineStr">
+    <row r="49">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>Historique antérieur au 2026-09-18 : voir worklog.md (racine du dépôt, versionné) — Tasks 1-41 (Identificateur, Backoffice, Supabase, voix offline, APK, fix CSP).</t>
         </is>

</xml_diff>

<commit_message>
fix(vocal): vente rapide — factory STT + watchdog (P0-1), montant dicté fait loi (P0-2), wake-word pause fiable, intents/confirmation (VOCAL-602..605, 628/628)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -3729,13 +3729,13 @@
           <t>AGENT 1</t>
         </is>
       </c>
-      <c r="H40" s="7" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+      <c r="H40" s="12" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
         </is>
       </c>
       <c r="I40" s="9" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
@@ -3749,12 +3749,12 @@
       </c>
       <c r="L40" s="7" t="inlineStr">
         <is>
-          <t>vente-rapide-modal.tsx, stt-factory.ts (helper partagé)</t>
+          <t>vente-rapide-modal.tsx, stt-factory.ts (startSmartSingleShotSTT nouveau)</t>
         </is>
       </c>
       <c r="M40" s="7" t="inlineStr">
         <is>
-          <t>Tests machine à états + choix moteur</t>
+          <t>5 tests session hybride (sync web, natif Sherpa, abort avant/après, erreur explicite) · 628/628 · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N40" s="7" t="inlineStr">
@@ -3781,7 +3781,7 @@
       <c r="S40" s="7" t="inlineStr"/>
       <c r="T40" s="7" t="inlineStr">
         <is>
-          <t>Corrige le spinner infini constaté sur APK ; donne le routage Baoulé gratuitement</t>
+          <t>LIVRÉ Task 54 : porte canAttemptSTT, session hybride sync-web/async-natif, watchdog 15 s, génération + abort ; smoke APK = B1-010/B5-052</t>
         </is>
       </c>
     </row>
@@ -3816,13 +3816,13 @@
           <t>AGENT 1</t>
         </is>
       </c>
-      <c r="H41" s="4" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+      <c r="H41" s="11" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
         </is>
       </c>
       <c r="I41" s="6" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
@@ -3836,12 +3836,12 @@
       </c>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>vente-rapide-modal.tsx, localIntent.ts</t>
+          <t>quick-sale.ts (planQuickSale nouveau + total dicté), localIntent.ts, vente-rapide-modal.tsx, voice-modal.tsx</t>
         </is>
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>4 scénarios chiffrés de l'audit §P0-2 en tests unitaires</t>
+          <t>11 tests quick-sale (4 scénarios audit + survente + timeout/file/stock) · 628/628 · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N41" s="4" t="inlineStr">
@@ -3868,7 +3868,7 @@
       <c r="S41" s="4" t="inlineStr"/>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>Impact métier direct : caisse/ventes/objectifs faussés silencieusement</t>
+          <t>LIVRÉ Task 54 : montant dicté fait loi + « à Y » nu = prix unitaire (total = qty × prix) + fin du vol de montant par priceUnit dans les 2 modales</t>
         </is>
       </c>
     </row>
@@ -3903,13 +3903,13 @@
           <t>AGENT 1</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+      <c r="H42" s="12" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
         </is>
       </c>
       <c r="I42" s="9" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
@@ -3923,12 +3923,12 @@
       </c>
       <c r="L42" s="7" t="inlineStr">
         <is>
-          <t>vente-rapide-modal.tsx, wake-word.ts, quick-sale.ts</t>
+          <t>vente-rapide-modal.tsx, wake-word.ts, quick-sale.ts, http.ts (nouveau)</t>
         </is>
       </c>
       <c r="M42" s="7" t="inlineStr">
         <is>
-          <t>Test : fetch suspendu → erreur à 10 s + file offline</t>
+          <t>3 tests wake-word pause + timeout 10 s → file offline · 628/628 · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N42" s="7" t="inlineStr">
@@ -3955,7 +3955,7 @@
       <c r="S42" s="7" t="inlineStr"/>
       <c r="T42" s="7" t="inlineStr">
         <is>
-          <t>fetchJsonWithTimeout déjà disponible (B4-041)</t>
+          <t>LIVRÉ Task 54 : _paused annule un start en vol (4 modales fixes), fetchJsonWithTimeout extrait dans http.ts (ré-export conversation.ts), stock après verdict, synced annoncé</t>
         </is>
       </c>
     </row>
@@ -3990,13 +3990,13 @@
           <t>AGENT 1</t>
         </is>
       </c>
-      <c r="H43" s="4" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+      <c r="H43" s="11" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
         </is>
       </c>
       <c r="I43" s="6" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
@@ -4010,12 +4010,12 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>vente-rapide-modal.tsx, localIntent.ts</t>
+          <t>vente-rapide-modal.tsx, localIntent.ts (AMOUNT_PATTERNS retiré), confirmations.ts (routeConfirmResponse nouveau)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>Parcours oui/stop/mes ventes/combien testés</t>
+          <t>6 tests routeConfirmResponse · 628/628 · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
@@ -4042,7 +4042,7 @@
       <c r="S43" s="4" t="inlineStr"/>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>Barge-in + prompts bci arbitrés séparément</t>
+          <t>LIVRÉ Task 54 : oui=écoute, stop ferme, navigation exécutée, consultation=total réel, confirmation=clavier sur erreur micro + enchaînement vente, dead code retiré, « D'accord » corrigé</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(vocal): mot de réveil — cycle de vie fiable : génération anti-double-session, réglage respecté (setWakeWordEnabled), pause tue le timer 10 s, stop sans zombie (VOCAL-606, 636/636)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -123,6 +123,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -488,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:T49"/>
+  <dimension ref="A2:T50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4049,60 +4050,60 @@
     <row r="44" ht="22" customHeight="1">
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>INF-401</t>
+          <t>VOCAL-606</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Audit vocal</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Déploiement prod + APK</t>
+          <t>Mot de réveil — cycle de vie fiable</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>Vercel puis APK autonome</t>
+          <t>Génération, réglage, pause timer, stop en vol</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
+          <t>Suite de la vérification « mot de réveil correctement implémenté » : 4 défauts trouvés et corrigés — F1 double resume à la fermeture de modale (body + cleanup d'effet) créait deux sessions concurrentes dont une orpheline à l'écoute → compteur de génération dans startWakeWordListener, le supplanté avorte ce qu'il vient de créer ; F2 resumeWakeWord ignorait le réglage wakeWordEnabled (fermer une modale rallumait le micro de fond désactivé) → setWakeWordEnabled piloté par WakeWordManager, resume bloqué si désactivé ; F3 la pause n'annulait ni le timer « retour à l'écoute » (10 s) ni l'état 'detected' — une modale ouverte &gt;10 s voyait le micro de fond ressusciter au milieu d'une vente → pauseWakeWord annule _resetTimer et nettoie l'état + garde _paused dans le timer ; F4 stop (logout) pendant un start en vol → session zombie → stop bump la génération. Cleanups conditionnels alignés sur voice-modal / prod-voice-modal / open-caisse-modal (même motif audité vente-rapide VOCAL-604).</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>ORCHESTRATEUR</t>
-        </is>
-      </c>
-      <c r="H44" s="7" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H44" s="12" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
         </is>
       </c>
       <c r="I44" s="9" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K44" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VOCAL-601</t>
         </is>
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
-          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
+          <t>wake-word.ts, wake-word-manager.tsx, voice-modal.tsx, prod-voice-modal.tsx, open-caisse-modal.tsx</t>
         </is>
       </c>
       <c r="M44" s="7" t="inlineStr">
         <is>
-          <t>Smoke APK</t>
+          <t>8 tests wake-word-lifecycle (nouveau : F1/F2/F3/F3b/F4 + détection/bruit) + 3 pause · 636/636 · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N44" s="7" t="inlineStr">
@@ -4118,55 +4119,55 @@
       </c>
       <c r="Q44" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="R44" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="S44" s="7" t="inlineStr"/>
       <c r="T44" s="7" t="inlineStr">
         <is>
-          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+          <t>LIVRÉ Task 55 : génération + _enabled + pause timer ; smoke device « Julaba » sur APK rejoint B1-010/B5-052</t>
         </is>
       </c>
     </row>
     <row r="45" ht="22" customHeight="1">
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>SEC-402</t>
+          <t>INF-401</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>PAT GitHub exposé</t>
+          <t>Déploiement prod + APK</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Révocation</t>
+          <t>Vercel puis APK autonome</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>USER</t>
-        </is>
-      </c>
-      <c r="H45" s="10" t="inlineStr">
-        <is>
-          <t>BLOQUÉ</t>
+          <t>ORCHESTRATEUR</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
         </is>
       </c>
       <c r="I45" s="6" t="n">
@@ -4174,7 +4175,7 @@
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K45" s="4" t="inlineStr">
@@ -4184,12 +4185,12 @@
       </c>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Smoke APK</t>
         </is>
       </c>
       <c r="N45" s="4" t="inlineStr">
@@ -4216,21 +4217,108 @@
       <c r="S45" s="4" t="inlineStr"/>
       <c r="T45" s="4" t="inlineStr">
         <is>
+          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>SEC-402</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>PAT GitHub exposé</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>Révocation</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="H46" s="13" t="inlineStr">
+        <is>
+          <t>BLOQUÉ</t>
+        </is>
+      </c>
+      <c r="I46" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K46" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L46" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M46" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N46" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O46" s="7" t="inlineStr"/>
+      <c r="P46" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q46" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="R46" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="S46" s="7" t="inlineStr"/>
+      <c r="T46" s="7" t="inlineStr">
+        <is>
           <t>Action utilisateur requise — P0 absolu</t>
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47"/>
-    <row r="48">
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
-        </is>
-      </c>
-    </row>
+    <row r="48"/>
     <row r="49">
       <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Historique antérieur au 2026-09-18 : voir worklog.md (racine du dépôt, versionné) — Tasks 1-41 (Identificateur, Backoffice, Supabase, voix offline, APK, fix CSP).</t>
         </is>

</xml_diff>

<commit_message>
ui(auth): première vue (numéro) restylée à l'identique de la maquette utilisateur — pill marché actif, avatar cerclé, carte connexion étal, champ paires + drapeau CI CSS, CTA gradient, barre d'écoute sombre (UI-701, 636/636)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -123,7 +123,6 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:T50"/>
+  <dimension ref="A2:T51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4137,41 +4136,41 @@
     <row r="45" ht="22" customHeight="1">
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>INF-401</t>
+          <t>UI-701</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Interface</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Déploiement prod + APK</t>
+          <t>Première vue — maquette « Connexion à votre étal »</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Vercel puis APK autonome</t>
+          <t>Vue numéro restylée d'après la maquette utilisateur</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
+          <t>Maquette fournie par l'utilisateur (capture) reproduite exactement sur la première vue (étape « name » de auth-screen) : barre supérieure (pill sombre « Mode marché actif » + pill blanc « Aide vocale » rejouant l'instruction Tata + sélecteur de rôle conservé), avatar circulaire cerclé d'orange avec badge boutique, pill « Caisse autonome &amp; 100% hors-ligne », titre Jùlaba sombre + sous-titre orange espacé, carte connexion (verrou orange, label majuscule, champ pill cerclé d'orange : drapeau CI rendu en CSS + +225 + saisie formatée en paires « 07 08 45 12 34 » + micro rond orange), CTA gradient « Continuer → », carte Assistance Vocale Tata réutilisée (icône Play, titre sur une ligne), lien « Nouvel étal ? S'enregistrer auprès du délégué » (Tata explique vocalement), barre d'écoute sombre fixe « Tata vous écoute... » pendant la dictée. Fonctionnel intact : normalisation soumission, dictée STT, note micro indisponible, erreurs, soleilMode.</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>ORCHESTRATEUR</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
         </is>
       </c>
       <c r="I45" s="6" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
@@ -4185,12 +4184,12 @@
       </c>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
+          <t>auth-screen.tsx (vue name + barre supérieure + tataCard resserrée)</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr">
         <is>
-          <t>Smoke APK</t>
+          <t>Rendu vérifié navigateur headless (captures vide/saisie) · 636/636 · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N45" s="4" t="inlineStr">
@@ -4206,55 +4205,55 @@
       </c>
       <c r="Q45" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="R45" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="S45" s="4" t="inlineStr"/>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+          <t>LIVRÉ Task 56 : formatage paires, drapeau CI en CSS (règle no-emoji), micro rond orange affiché si micro dispo ; smoke dictée sur device rejoint B1-010/B5-052</t>
         </is>
       </c>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>SEC-402</t>
+          <t>INF-401</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>PAT GitHub exposé</t>
+          <t>Déploiement prod + APK</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>Révocation</t>
+          <t>Vercel puis APK autonome</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>USER</t>
-        </is>
-      </c>
-      <c r="H46" s="13" t="inlineStr">
-        <is>
-          <t>BLOQUÉ</t>
+          <t>ORCHESTRATEUR</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
         </is>
       </c>
       <c r="I46" s="9" t="n">
@@ -4262,7 +4261,7 @@
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K46" s="7" t="inlineStr">
@@ -4272,12 +4271,12 @@
       </c>
       <c r="L46" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
         </is>
       </c>
       <c r="M46" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Smoke APK</t>
         </is>
       </c>
       <c r="N46" s="7" t="inlineStr">
@@ -4304,21 +4303,108 @@
       <c r="S46" s="7" t="inlineStr"/>
       <c r="T46" s="7" t="inlineStr">
         <is>
+          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>SEC-402</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>PAT GitHub exposé</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Révocation</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="H47" s="10" t="inlineStr">
+        <is>
+          <t>BLOQUÉ</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N47" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O47" s="4" t="inlineStr"/>
+      <c r="P47" s="4" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q47" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="R47" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="S47" s="4" t="inlineStr"/>
+      <c r="T47" s="4" t="inlineStr">
+        <is>
           <t>Action utilisateur requise — P0 absolu</t>
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48"/>
-    <row r="49">
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
-        </is>
-      </c>
-    </row>
+    <row r="49"/>
     <row r="50">
       <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>Historique antérieur au 2026-09-18 : voir worklog.md (racine du dépôt, versionné) — Tasks 1-41 (Identificateur, Backoffice, Supabase, voix offline, APK, fix CSP).</t>
         </is>

</xml_diff>

<commit_message>
feat(vocal): comportement conversationnel de Tata — résumé vocal du jour sur données réelles (serveur + file offline + repli agrégats), confirmations détaillées sans formule de fin, fin de conversation explicite intent end (VOCAL-607, 676/676)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -123,6 +123,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -488,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:T51"/>
+  <dimension ref="A2:T52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4223,60 +4224,60 @@
     <row r="46" ht="22" customHeight="1">
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>INF-401</t>
+          <t>VOCAL-607</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Audit vocal</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Déploiement prod + APK</t>
+          <t>Comportement conversationnel de Tata</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>Vercel puis APK autonome</t>
+          <t>Résumé vocal du jour, fin de conversation, confirmations détaillées</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
+          <t>Demande utilisateur : comportement conversationnel et contextuel, plus de formule de fin récitée — (1) Résumé vocal du jour : la tuile « Résumé du jour » dicte TOUTES les ventes réelles de la journée (produit, quantité, montant par vente) puis le total, à partir des données réelles (serveur + file offline fusionnées, repli agrégats caisse), « Tu n'as encore enregistré aucune vente aujourd'hui. » si vide, jamais de vente/prix inventé, bouton « Écouter le détail des ventes » dans la modale ; (2) après une vente enregistrée : confirmation détaillée « Vente enregistrée : 2 sacs de riz pour 25 000 francs. » (+ notes sync/stock) SANS « Bonne journée », Tata ré-écoute et attend la vente suivante ; (3) fin de conversation : nouvel intent 'end' (« c'est tout », « j'ai fini », « au revoir », « plus rien à faire », « à demain »…) → « D'accord, à bientôt et bonne journée ! » unique (TATA_GOODBYE), « plus rien » retiré du cancel ; (4) consultation vocale dans la modale générale = vrai total du jour (fini le mensonger « Consultation en cours... »). Logique d'enregistrement des ventes INTACTE (quick-sale, stock, caisse).</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>ORCHESTRATEUR</t>
-        </is>
-      </c>
-      <c r="H46" s="7" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H46" s="12" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
         </is>
       </c>
       <c r="I46" s="9" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K46" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VOCAL-601</t>
         </is>
       </c>
       <c r="L46" s="7" t="inlineStr">
         <is>
-          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
+          <t>localIntent.ts (intent end + TATA_GOODBYE), tata-phrases.ts (nouveau), day-summary.ts (nouveau), vente-rapide-modal.tsx, voice-modal.tsx, home-screen.tsx</t>
         </is>
       </c>
       <c r="M46" s="7" t="inlineStr">
         <is>
-          <t>Smoke APK</t>
+          <t>24 tests (10 tata-phrases + 14 day-summary) + 17 tests intent end · 676/676 (45 fichiers) · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N46" s="7" t="inlineStr">
@@ -4292,55 +4293,55 @@
       </c>
       <c r="Q46" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="R46" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="S46" s="7" t="inlineStr"/>
       <c r="T46" s="7" t="inlineStr">
         <is>
-          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+          <t>LIVRÉ Task 57 : dicté fidèle aux données réelles (total dicté fait loi sur la ligne), plafond honnête à 12 lignes dictées puis « et N autres ventes » avec total réel complet ; smoke device rejoint B1-010/B5-052</t>
         </is>
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>SEC-402</t>
+          <t>INF-401</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>PAT GitHub exposé</t>
+          <t>Déploiement prod + APK</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Révocation</t>
+          <t>Vercel puis APK autonome</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>USER</t>
-        </is>
-      </c>
-      <c r="H47" s="10" t="inlineStr">
-        <is>
-          <t>BLOQUÉ</t>
+          <t>ORCHESTRATEUR</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
         </is>
       </c>
       <c r="I47" s="6" t="n">
@@ -4348,7 +4349,7 @@
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K47" s="4" t="inlineStr">
@@ -4358,12 +4359,12 @@
       </c>
       <c r="L47" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
         </is>
       </c>
       <c r="M47" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Smoke APK</t>
         </is>
       </c>
       <c r="N47" s="4" t="inlineStr">
@@ -4390,21 +4391,108 @@
       <c r="S47" s="4" t="inlineStr"/>
       <c r="T47" s="4" t="inlineStr">
         <is>
+          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>SEC-402</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>PAT GitHub exposé</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>Révocation</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="H48" s="13" t="inlineStr">
+        <is>
+          <t>BLOQUÉ</t>
+        </is>
+      </c>
+      <c r="I48" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K48" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L48" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M48" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N48" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O48" s="7" t="inlineStr"/>
+      <c r="P48" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q48" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="R48" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="S48" s="7" t="inlineStr"/>
+      <c r="T48" s="7" t="inlineStr">
+        <is>
           <t>Action utilisateur requise — P0 absolu</t>
         </is>
       </c>
     </row>
-    <row r="48"/>
     <row r="49"/>
-    <row r="50">
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
-        </is>
-      </c>
-    </row>
+    <row r="50"/>
     <row r="51">
       <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>Historique antérieur au 2026-09-18 : voir worklog.md (racine du dépôt, versionné) — Tasks 1-41 (Identificateur, Backoffice, Supabase, voix offline, APK, fix CSP).</t>
         </is>

</xml_diff>

<commit_message>
feat(vocal): le résumé du jour dicte aussi les dépenses réelles — serveur /api/marchand/expenses + file offline + repli agrégat todayExpenses, dicté « Tu as aussi dépensé X francs pour … » + total, bilan vide « aucune vente ni dépense », jamais inventé, logique d'enregistrement intacte (VOCAL-608, 685/685)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -123,7 +123,6 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:T52"/>
+  <dimension ref="A2:T53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4311,60 +4310,60 @@
     <row r="47" ht="22" customHeight="1">
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>INF-401</t>
+          <t>VOCAL-608</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Audit vocal</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Déploiement prod + APK</t>
+          <t>Résumé du jour — dépenses dictées</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Vercel puis APK autonome</t>
+          <t>Tata dicte AUSSI les dépenses réelles du jour</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
+          <t>Demande utilisateur : « je veux aussi que Tata dicte aussi les dépenses du jour dans ce résumé ». Extension du résumé vocal du jour (VOCAL-607) : collecte des dépenses réelles du jour (serveur /api/marchand/expenses?merchantId&amp;startDate&amp;endDate borné 6 s + file offline fusionnée — une dépense en file n'a jamais atteint le serveur, pas de doublon —, repli INDÉPENDANT sur l'agrégat todayExpenses du store caisse, symétrique aux ventes) ; dicté après les ventes : chaque dépense « Tu as aussi dépensé 1 000 francs pour Transport et 500 francs pour Aliment. Au total, tes dépenses s'élèvent à 1 500 francs. », libellé = description réelle enregistrée sinon libellé FR de la catégorie (EXPENSE_CATEGORY_LABELS aligné écran Dépenses) sinon catégorie brute — JAMAIS fabriqué ; « Tu n'as enregistré aucune dépense aujourd'hui. » si vide ; bilan vide couvrant les deux « aucune vente ni dépense aujourd'hui » ; repli agrégats « Tes dépenses du jour s'élèvent à X francs. » sans détail inventé ; plafond honnête 12 lignes puis « et N autres dépenses », total réel complet. Intro « Un instant, je regarde tes ventes et tes dépenses du jour. ». Logique d'enregistrement des ventes ET dépenses INTACTE (lecture seule).</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>ORCHESTRATEUR</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
         </is>
       </c>
       <c r="I47" s="6" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K47" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VOCAL-607</t>
         </is>
       </c>
       <c r="L47" s="4" t="inlineStr">
         <is>
-          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
+          <t>day-summary.ts (collecte + dicté dépenses), home-screen.tsx (intro)</t>
         </is>
       </c>
       <c r="M47" s="4" t="inlineStr">
         <is>
-          <t>Smoke APK</t>
+          <t>9 tests nouveaux (day-summary 23) · 685/685 (45 fichiers) · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N47" s="4" t="inlineStr">
@@ -4380,55 +4379,55 @@
       </c>
       <c r="Q47" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="R47" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="S47" s="4" t="inlineStr"/>
       <c r="T47" s="4" t="inlineStr">
         <is>
-          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+          <t>LIVRÉ Task 58 : champs dépenses optionnels (dicté VOCAL-607 inchangé pour anciens appelants), sources réelles uniquement ; smoke device rejoint B1-010/B5-052</t>
         </is>
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>SEC-402</t>
+          <t>INF-401</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>PAT GitHub exposé</t>
+          <t>Déploiement prod + APK</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>Révocation</t>
+          <t>Vercel puis APK autonome</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>USER</t>
-        </is>
-      </c>
-      <c r="H48" s="13" t="inlineStr">
-        <is>
-          <t>BLOQUÉ</t>
+          <t>ORCHESTRATEUR</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
         </is>
       </c>
       <c r="I48" s="9" t="n">
@@ -4436,7 +4435,7 @@
       </c>
       <c r="J48" s="7" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K48" s="7" t="inlineStr">
@@ -4446,12 +4445,12 @@
       </c>
       <c r="L48" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
         </is>
       </c>
       <c r="M48" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Smoke APK</t>
         </is>
       </c>
       <c r="N48" s="7" t="inlineStr">
@@ -4478,21 +4477,108 @@
       <c r="S48" s="7" t="inlineStr"/>
       <c r="T48" s="7" t="inlineStr">
         <is>
+          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>SEC-402</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>PAT GitHub exposé</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Révocation</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="H49" s="10" t="inlineStr">
+        <is>
+          <t>BLOQUÉ</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M49" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N49" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O49" s="4" t="inlineStr"/>
+      <c r="P49" s="4" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q49" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="R49" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="S49" s="4" t="inlineStr"/>
+      <c r="T49" s="4" t="inlineStr">
+        <is>
           <t>Action utilisateur requise — P0 absolu</t>
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50"/>
-    <row r="51">
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
-        </is>
-      </c>
-    </row>
+    <row r="51"/>
     <row r="52">
       <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>Historique antérieur au 2026-09-18 : voir worklog.md (racine du dépôt, versionné) — Tasks 1-41 (Identificateur, Backoffice, Supabase, voix offline, APK, fix CSP).</t>
         </is>

</xml_diff>

<commit_message>
feat(vocal): solde de caisse (ventes − dépenses) dicté en toute fin du résumé du jour — « Ton solde de caisse pour aujourd'hui est de X francs. », cas négatif honnête « tes dépenses dépassent tes ventes », pas de solde sur jour vide, gate rétrocompat VOCAL-607 (VOCAL-609, 689/689)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -123,6 +123,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -488,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:T53"/>
+  <dimension ref="A2:T54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4397,41 +4398,41 @@
     <row r="48" ht="22" customHeight="1">
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>INF-401</t>
+          <t>VOCAL-609</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Audit vocal</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Déploiement prod + APK</t>
+          <t>Résumé du jour — solde de caisse</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>Vercel puis APK autonome</t>
+          <t>Solde ventes − dépenses dicté en fin de résumé</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
+          <t>Demande utilisateur : « Tata annonce le solde de caisse (ventes − dépenses) en fin de résumé ». soldePart(data) ajouté EN FIN du dicté du résumé : « Ton solde de caisse pour aujourd'hui est de X francs. » ; formule demandée = VENTES − DÉPENSES (le fond de caisse n'entre PAS dans ce dicté — le bouton « balance » de l'accueil reste la référence caisse complète avec fond) ; solde négatif dit honnêtement « Attention, tes dépenses dépassent tes ventes de X francs. » (jamais « moins X francs » que le TTS lirait mal) ; jour totalement vide → PAS de solde dicté (bilan vide seulement) ; gate sur les champs dépenses (rétrocompatibilité VOCAL-607 : sans champs → dicté strict sans solde) ; repli agrégats = solde calculé depuis les TOTAUX réels persistés. Logique d'enregistrement INTACTE (lecture seule).</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>ORCHESTRATEUR</t>
-        </is>
-      </c>
-      <c r="H48" s="7" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H48" s="12" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
         </is>
       </c>
       <c r="I48" s="9" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J48" s="7" t="inlineStr">
         <is>
@@ -4440,17 +4441,17 @@
       </c>
       <c r="K48" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VOCAL-608</t>
         </is>
       </c>
       <c r="L48" s="7" t="inlineStr">
         <is>
-          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
+          <t>day-summary.ts (soldePart + assemblage du dicté), home-screen.tsx (commentaire)</t>
         </is>
       </c>
       <c r="M48" s="7" t="inlineStr">
         <is>
-          <t>Smoke APK</t>
+          <t>4 tests nouveaux (day-summary 27 : solde en fin, ventes=dépenses → 0, rétrocompat sans solde, repli agrégats) · 689/689 (45 fichiers) · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N48" s="7" t="inlineStr">
@@ -4466,55 +4467,55 @@
       </c>
       <c r="Q48" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="R48" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="S48" s="7" t="inlineStr"/>
       <c r="T48" s="7" t="inlineStr">
         <is>
-          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+          <t>LIVRÉ Task 59 : solde = données réelles uniquement, cas négatif et jour vide traités ; smoke device rejoint B1-010/B5-052</t>
         </is>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>SEC-402</t>
+          <t>INF-401</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>PAT GitHub exposé</t>
+          <t>Déploiement prod + APK</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Révocation</t>
+          <t>Vercel puis APK autonome</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>USER</t>
-        </is>
-      </c>
-      <c r="H49" s="10" t="inlineStr">
-        <is>
-          <t>BLOQUÉ</t>
+          <t>ORCHESTRATEUR</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
         </is>
       </c>
       <c r="I49" s="6" t="n">
@@ -4522,7 +4523,7 @@
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K49" s="4" t="inlineStr">
@@ -4532,12 +4533,12 @@
       </c>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
         </is>
       </c>
       <c r="M49" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Smoke APK</t>
         </is>
       </c>
       <c r="N49" s="4" t="inlineStr">
@@ -4564,21 +4565,108 @@
       <c r="S49" s="4" t="inlineStr"/>
       <c r="T49" s="4" t="inlineStr">
         <is>
+          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>SEC-402</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>PAT GitHub exposé</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Révocation</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="H50" s="13" t="inlineStr">
+        <is>
+          <t>BLOQUÉ</t>
+        </is>
+      </c>
+      <c r="I50" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K50" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L50" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M50" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N50" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O50" s="7" t="inlineStr"/>
+      <c r="P50" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q50" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="R50" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="S50" s="7" t="inlineStr"/>
+      <c r="T50" s="7" t="inlineStr">
+        <is>
           <t>Action utilisateur requise — P0 absolu</t>
         </is>
       </c>
     </row>
-    <row r="50"/>
     <row r="51"/>
-    <row r="52">
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
-        </is>
-      </c>
-    </row>
+    <row r="52"/>
     <row r="53">
       <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>Historique antérieur au 2026-09-18 : voir worklog.md (racine du dépôt, versionné) — Tasks 1-41 (Identificateur, Backoffice, Supabase, voix offline, APK, fix CSP).</t>
         </is>

</xml_diff>

<commit_message>
feat(vocal): formulation du dicté du résumé ajustée au registre parlé — « En tout, ça fait 3 ventes pour 34 500 francs. », « Tes dépenses font X francs. », solde « Ton solde de caisse est de X francs. » (« zéro franc » si nul), transition « Tu as aussi dépensé » réservée aux journées avec ventes, zéro changement de fond (VOCAL-610, 691/691)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -123,7 +123,6 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:T54"/>
+  <dimension ref="A2:T55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4485,41 +4484,41 @@
     <row r="49" ht="22" customHeight="1">
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>INF-401</t>
+          <t>VOCAL-610</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Audit vocal</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Déploiement prod + APK</t>
+          <t>Résumé du jour — formulation orale</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Vercel puis APK autonome</t>
+          <t>Formulation du dicté ajustée (registre parlé)</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
+          <t>Demande utilisateur : « ajuster la formulation du dicté ». Passe de style sur le dicté du résumé du jour (ventes + dépenses + solde), ZÉRO changement de fond — mêmes données réelles, plafond 12 lignes, total complet jamais tronqué, rétrocompatibilité : total ventes « En tout, ça fait 3 ventes pour 34 500 francs. » (fini « Au total, tu as réalisé … pour un montant de ») ; repli agrégats ventes « Aujourd'hui, tu as fait 2 ventes pour 9 000 francs. » ; total dépenses « Tes dépenses font 1 500 francs. » (fini « Au total, tes dépenses s'élèvent à » — « Au total » n'apparaît plus deux fois dans le même dicté) ; repli agrégats dépenses aligné « Tes dépenses font X francs. » ; transition « Tu as AUSSI dépensé » réservée aux journées avec ventes (sans vente : « Tu as dépensé … » — transition jamais orpheline) ; solde « Ton solde de caisse est de X francs. » (fini « pour aujourd'hui », redondant dans un résumé du jour) et solde nul dicté « zéro franc » ; cas négatif inchangé (« Attention, tes dépenses dépassent tes ventes de X francs. »). Logique d'enregistrement INTACTE (lecture seule).</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>ORCHESTRATEUR</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H49" s="11" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
         </is>
       </c>
       <c r="I49" s="6" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
@@ -4528,17 +4527,17 @@
       </c>
       <c r="K49" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VOCAL-609</t>
         </is>
       </c>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
+          <t>day-summary.ts (formulations ventes/dépenses/solde), day-summary.test.ts</t>
         </is>
       </c>
       <c r="M49" s="4" t="inlineStr">
         <is>
-          <t>Smoke APK</t>
+          <t>2 tests nouveaux (day-summary 29 : bannissement du registre écrit, transition « aussi » réservée aux ventes) · 691/691 (45 fichiers) · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N49" s="4" t="inlineStr">
@@ -4554,55 +4553,55 @@
       </c>
       <c r="Q49" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="R49" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="S49" s="4" t="inlineStr"/>
       <c r="T49" s="4" t="inlineStr">
         <is>
-          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+          <t>LIVRÉ Task 60 : français parlé naturel à l'oreille, tous les invariants conservés ; smoke device rejoint B1-010/B5-052</t>
         </is>
       </c>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>SEC-402</t>
+          <t>INF-401</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>PAT GitHub exposé</t>
+          <t>Déploiement prod + APK</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>Révocation</t>
+          <t>Vercel puis APK autonome</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>USER</t>
-        </is>
-      </c>
-      <c r="H50" s="13" t="inlineStr">
-        <is>
-          <t>BLOQUÉ</t>
+          <t>ORCHESTRATEUR</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
         </is>
       </c>
       <c r="I50" s="9" t="n">
@@ -4610,7 +4609,7 @@
       </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K50" s="7" t="inlineStr">
@@ -4620,12 +4619,12 @@
       </c>
       <c r="L50" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
         </is>
       </c>
       <c r="M50" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Smoke APK</t>
         </is>
       </c>
       <c r="N50" s="7" t="inlineStr">
@@ -4652,21 +4651,108 @@
       <c r="S50" s="7" t="inlineStr"/>
       <c r="T50" s="7" t="inlineStr">
         <is>
+          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>SEC-402</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>PAT GitHub exposé</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>Révocation</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="H51" s="10" t="inlineStr">
+        <is>
+          <t>BLOQUÉ</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M51" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N51" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O51" s="4" t="inlineStr"/>
+      <c r="P51" s="4" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q51" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="R51" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="S51" s="4" t="inlineStr"/>
+      <c r="T51" s="4" t="inlineStr">
+        <is>
           <t>Action utilisateur requise — P0 absolu</t>
         </is>
       </c>
     </row>
-    <row r="51"/>
     <row r="52"/>
-    <row r="53">
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
-        </is>
-      </c>
-    </row>
+    <row r="53"/>
     <row r="54">
       <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>Historique antérieur au 2026-09-18 : voir worklog.md (racine du dépôt, versionné) — Tasks 1-41 (Identificateur, Backoffice, Supabase, voix offline, APK, fix CSP).</t>
         </is>

</xml_diff>

<commit_message>
feat(vocal): solde dicté « Il te reste X francs en caisse. » — formulation orale choisie par l'utilisatrice, solde nul « Il ne te reste plus rien en caisse. », négatif inchangé honnête, zéro changement de fond (VOCAL-611, 694/694)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -123,6 +123,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -488,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:T55"/>
+  <dimension ref="A2:T56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4571,41 +4572,41 @@
     <row r="50" ht="22" customHeight="1">
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>INF-401</t>
+          <t>VOCAL-611</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Audit vocal</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Déploiement prod + APK</t>
+          <t>Résumé du jour — formulation du solde</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>Vercel puis APK autonome</t>
+          <t>Solde dicté « Il te reste X francs en caisse »</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
+          <t>Choix de formulation de l'utilisatrice : « Il te reste X francs en caisse » remplace « Ton solde de caisse est de X francs. » pour la phrase de solde (VOCAL-609) — zéro changement de fond. soldePart() : solde positif « Il te reste X francs en caisse. » (montantParle + francs, DERNIÈRE phrase du dicté) ; solde nul « Il ne te reste plus rien en caisse. » (naturel à l'oreille, fini « zéro franc » plaqué) ; solde négatif inchangé « Attention, tes dépenses dépassent tes ventes de X francs. » (« Il te reste » n'a pas de sens en dessous de zéro) ; jour totalement vide → toujours PAS de solde ; gate rétrocompatibilité VOCAL-607 intact (sans champs dépenses → aucun solde). Formule VENTES − DÉPENSES inchangée, fond de caisse toujours exclu, données réelles uniquement, plafond 12 lignes, logique d'enregistrement INTACTE (lecture seule).</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>ORCHESTRATEUR</t>
-        </is>
-      </c>
-      <c r="H50" s="7" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H50" s="12" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
         </is>
       </c>
       <c r="I50" s="9" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
@@ -4614,17 +4615,17 @@
       </c>
       <c r="K50" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VOCAL-610</t>
         </is>
       </c>
       <c r="L50" s="7" t="inlineStr">
         <is>
-          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
+          <t>day-summary.ts (soldePart + doc), day-summary.test.ts</t>
         </is>
       </c>
       <c r="M50" s="7" t="inlineStr">
         <is>
-          <t>Smoke APK</t>
+          <t>3 tests nouveaux (day-summary 32 : solde positif formulation demandée en fin de dicté, solde nul naturel, solde négatif honnête sans « Il te reste ») · 694/694 (45 fichiers) · tsc 0 · lint 0 · build prod OK</t>
         </is>
       </c>
       <c r="N50" s="7" t="inlineStr">
@@ -4640,55 +4641,55 @@
       </c>
       <c r="Q50" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="R50" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="S50" s="7" t="inlineStr"/>
       <c r="T50" s="7" t="inlineStr">
         <is>
-          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+          <t>LIVRÉ Task 61 : formulation orale choisie par l'utilisatrice, tous les invariants conservés ; smoke device rejoint B1-010/B5-052</t>
         </is>
       </c>
     </row>
     <row r="51" ht="22" customHeight="1">
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>SEC-402</t>
+          <t>INF-401</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>PAT GitHub exposé</t>
+          <t>Déploiement prod + APK</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Révocation</t>
+          <t>Vercel puis APK autonome</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>USER</t>
-        </is>
-      </c>
-      <c r="H51" s="10" t="inlineStr">
-        <is>
-          <t>BLOQUÉ</t>
+          <t>ORCHESTRATEUR</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
         </is>
       </c>
       <c r="I51" s="6" t="n">
@@ -4696,7 +4697,7 @@
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K51" s="4" t="inlineStr">
@@ -4706,12 +4707,12 @@
       </c>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
         </is>
       </c>
       <c r="M51" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Smoke APK</t>
         </is>
       </c>
       <c r="N51" s="4" t="inlineStr">
@@ -4738,21 +4739,108 @@
       <c r="S51" s="4" t="inlineStr"/>
       <c r="T51" s="4" t="inlineStr">
         <is>
+          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>SEC-402</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>PAT GitHub exposé</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>Révocation</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="H52" s="13" t="inlineStr">
+        <is>
+          <t>BLOQUÉ</t>
+        </is>
+      </c>
+      <c r="I52" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K52" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L52" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M52" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N52" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O52" s="7" t="inlineStr"/>
+      <c r="P52" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q52" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="R52" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="S52" s="7" t="inlineStr"/>
+      <c r="T52" s="7" t="inlineStr">
+        <is>
           <t>Action utilisateur requise — P0 absolu</t>
         </is>
       </c>
     </row>
-    <row r="52"/>
     <row r="53"/>
-    <row r="54">
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
-        </is>
-      </c>
-    </row>
+    <row r="54"/>
     <row r="55">
       <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Historique antérieur au 2026-09-18 : voir worklog.md (racine du dépôt, versionné) — Tasks 1-41 (Identificateur, Backoffice, Supabase, voix offline, APK, fix CSP).</t>
         </is>

</xml_diff>

<commit_message>
docs(stock): audit + plan du système de stock par mouvements (STK-801) — PHASE 1 audit lecture seule (DB/RLS/API, front/offline, vocal) + PHASE 2 plan (merchant_stock_*, RPC transactionnelles, refus strict stock insuffisant, OPENING_BALANCE, unités CI, offline operation_id, tests pgTAP) — aucun code applicatif modifié, registre 60 tâches (Task 62)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:T56"/>
+  <dimension ref="A2:T68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -507,7 +507,7 @@
     <col width="34" customWidth="1" min="13" max="13"/>
     <col width="34" customWidth="1" min="14" max="14"/>
     <col width="9" customWidth="1" min="15" max="15"/>
-    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
@@ -4659,45 +4659,45 @@
     <row r="51" ht="22" customHeight="1">
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>INF-401</t>
+          <t>STK-801</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Déploiement prod + APK</t>
+          <t>Audit + plan du système de stock</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Vercel puis APK autonome</t>
+          <t>Registre de mouvements fiable — audit + plan (sans code)</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
+          <t>PHASE 1 AUDIT : architecture (2 générations de tables : legacy actif service_role / moderne org-scoped orphelin), stock actuel = legacy_products.stock_qty décrémenté CLIENT-side en 3 points (quick-sale.ts:114, caisse-screen.tsx:139, voice-modal.tsx:194) sans CHECK ni journal, POST /api/marchand/sales sans toucher au stock, RPC create_sale transactionnelle SANS appelant, idempotence client_id réelle, 12 handlers offline, vocal : 13 intents sans intents stock, unités parsées limitées, écrêtage survente non bloquant. PHASE 2 PLAN : 7 décisions d'architecture (D1 construire sur flux actif, D2 legacy_sales conservé + RPC unique, D3 double écriture temporaire stock_qty/balance, D4 mouvements signés, D5 append-only, D6 perte ≠ dépense, D7 montant-sans-quantité → demande de quantité), schéma merchant_stock_* (units, prices, balances CHECK&gt;=0, movements 14 types append-only unique(merchant_id, operation_id)), purchases, transfers, business_partners, RPC transactionnelles avec erreurs métier JSON, backfill OPENING_BALANCE, refus strict stock insuffisant (remplace l'écrêtage), vocal intents stock + unités locales, offline operation_id + conflits, UI simple, tests vitest + pgTAP concurrence.</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>ORCHESTRATEUR</t>
-        </is>
-      </c>
-      <c r="H51" s="4" t="inlineStr">
-        <is>
-          <t>A_FAIRE</t>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I51" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K51" s="4" t="inlineStr">
@@ -4707,12 +4707,12 @@
       </c>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
+          <t>.ai/PLAN_STOCK.md (audit PHASE 1 + plan PHASE 2 complet)</t>
         </is>
       </c>
       <c r="M51" s="4" t="inlineStr">
         <is>
-          <t>Smoke APK</t>
+          <t>Audit en lecture seule (3 axes : DB/RLS/API, front/offline, vocal/ventes) · zéro code applicatif modifié (méthode §47) · plan soumis à validation utilisateur</t>
         </is>
       </c>
       <c r="N51" s="4" t="inlineStr">
@@ -4728,55 +4728,55 @@
       </c>
       <c r="Q51" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="R51" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="S51" s="4" t="inlineStr"/>
       <c r="T51" s="4" t="inlineStr">
         <is>
-          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+          <t>LIVRÉ Task 62 : 92 tables cartographiées, gaps identifiés (achats/fournisseurs/unités/intents stock/vérification serveur), plan + 11 tâches STK-802..812 créées</t>
         </is>
       </c>
     </row>
     <row r="52" ht="22" customHeight="1">
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>SEC-402</t>
+          <t>STK-802</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>PAT GitHub exposé</t>
+          <t>Migrations DB stock</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>Révocation</t>
+          <t>Tables merchant_stock_* + purchases + transfers + partners + backfill OPENING_BALANCE</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+          <t>Migrations SQL (1 objet = 1 fichier, convention dépôt) : merchant_product_units (unités locales kg/sac/carton/bassine/panier/tas/botte/bidon/fût/seau/pièce/litre…, conversion configurable par produit/marchand vers unité de base, un seul is_base), merchant_product_prices (PURCHASE/RETAIL/WHOLESALE/SEMI_WHOLESALE, validité temporelle), merchant_stock_balances (quantity_base numeric(14,3) CHECK &gt;= 0 — stock négatif physiquement impossible, stock_precision EXACT/ESTIMATED/UNKNOWN, low_stock_threshold paramétrable, weighted_avg_cost), merchant_stock_movements (journal APPEND-ONLY signé, 14 types OPENING_BALANCE/PURCHASE/RECEIPT/PRODUCTION/CUSTOMER_RETURN/TRANSFER_IN/ADJUSTMENT_IN/SALE/LOSS/DAMAGE/DONATION/SUPPLIER_RETURN/TRANSFER_OUT/ADJUSTMENT_OUT, reason, reference_id, device_id, UNIQUE(merchant_id, operation_id) — idempotence), merchant_purchases + items, merchant_stock_transfers + items (identifiant commun), business_partners (client/fournisseur). RLS activé default deny (régime service_role). Backfill : chaque legacy_products actif stock_qty&gt;0 → OPENING_BALANCE + balance EXACT (operation_id déterministe, rejouable). Anciennes données TOUTES conservées.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>USER</t>
-        </is>
-      </c>
-      <c r="H52" s="13" t="inlineStr">
-        <is>
-          <t>BLOQUÉ</t>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
         </is>
       </c>
       <c r="I52" s="9" t="n">
@@ -4784,17 +4784,17 @@
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K52" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>STK-801</t>
         </is>
       </c>
       <c r="L52" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>supabase/migrations/*.sql (1 table = 1 fichier), supabase/tests/rls.sql</t>
         </is>
       </c>
       <c r="M52" s="7" t="inlineStr">
@@ -4810,37 +4810,1057 @@
       <c r="O52" s="7" t="inlineStr"/>
       <c r="P52" s="7" t="inlineStr">
         <is>
-          <t>Aucune</t>
+          <t>Concurrence de nom évitée : préfixe merchant_stock_ (la table moderne stock_movements org-scoped existe)</t>
         </is>
       </c>
       <c r="Q52" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="R52" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="S52" s="7" t="inlineStr"/>
       <c r="T52" s="7" t="inlineStr">
         <is>
+          <t>Priorité 1 de la séquence d'implémentation §47</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>STK-803</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>RPC transactionnelles stock</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>record_sale / record_purchase / record_movement / adjust_to_count / transferts</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Fonctions PostgreSQL (1 fonction = 1 fichier) : merchant_record_sale (1. idempotence (merchant_id, operation_id) → retourne l'existant ; 2. SELECT…FOR UPDATE balance triée par product_id anti-deadlock ; 3. refus RAISE avec payload JSON INSUFFICIENT_STOCK {available, requested, unit, product} si requested &gt; available ; 4. INSERT legacy_sales + legacy_sale_items (total recalculé serveur) ; 5. mouvement SALE signé + UPDATE balance + double écriture legacy_products.stock_qty ; 6. COMMIT/ROLLBACK tout-ou-rien), merchant_record_purchase (achat + PURCHASE + balance + coût moyen pondéré), merchant_record_movement (LOSS/DAMAGE/DONATION/RETURN/PRODUCTION/RECEIPT/ADJUSTMENT_* avec reason obligatoire), merchant_adjust_to_count (comptage → delta → ADJUSTMENT_IN/OUT reason=INVENTORY_COUNT, jamais d'écrasement), merchant_transfer_out/receive (2 transactions liées par transfer_id). Erreurs métier explicites : INSUFFICIENT_STOCK, PRODUCT_NOT_FOUND, INVALID_QUANTITY, INVALID_UNIT, PRODUCT_INACTIVE, DUPLICATE_OPERATION, UNKNOWN_STOCK.</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K53" s="4" t="inlineStr">
+        <is>
+          <t>STK-802</t>
+        </is>
+      </c>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>supabase/migrations/*.sql (1 fonction = 1 fichier), supabase/tests/*.sql pgTAP</t>
+        </is>
+      </c>
+      <c r="M53" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N53" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O53" s="4" t="inlineStr"/>
+      <c r="P53" s="4" t="inlineStr">
+        <is>
+          <t>Modèle = create_sale moderne (20260908001730) adapté au flux marchand actif ; pgTAP concurrence 7+5 sur 10 → jamais −2</t>
+        </is>
+      </c>
+      <c r="Q53" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R53" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S53" s="4" t="inlineStr"/>
+      <c r="T53" s="4" t="inlineStr">
+        <is>
+          <t>La garantie « stock jamais négatif » vit ICI (serveur), pas dans React</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>STK-804</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>StockService + API</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>Couche service centralisée + routes /api/marchand/stock/* + bascule route ventes</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>src/lib/stock/stock-service.ts : getStock, checkAvailability, recordSale, recordPurchase, recordLoss, recordAdjustment, adjustToCount, createTransfer, receiveTransfer, getMovements + formatStockDisplay (affichage commercial « 2 sacs + 13 kg »). Routes : POST/GET /api/marchand/stock/movements, GET /api/marchand/stock/balance, POST/GET /api/marchand/purchases, POST/GET /api/marchand/stock/transfers, GET/POST /api/marchand/stock/units — toutes zod + requireDeviceOwner + mapping erreurs RPC (INSUFFICIENT_STOCK → 422 + {available, requested, unit}). POST /api/marchand/sales bascule sur la RPC merchant_record_sale (GET inchangé). ZÉRO duplication de logique métier dans les routes.</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I54" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K54" s="7" t="inlineStr">
+        <is>
+          <t>STK-803</t>
+        </is>
+      </c>
+      <c r="L54" s="7" t="inlineStr">
+        <is>
+          <t>src/lib/stock/stock-service.ts (nouveau), src/app/api/marchand/stock/** (nouveau), src/app/api/marchand/sales/route.ts, src/lib/validation/marchand.ts</t>
+        </is>
+      </c>
+      <c r="M54" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N54" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O54" s="7" t="inlineStr"/>
+      <c r="P54" s="7" t="inlineStr">
+        <is>
+          <t>La route ventes actuelle reste idempotente sur clientId (= operation_id)</t>
+        </is>
+      </c>
+      <c r="Q54" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R54" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S54" s="7" t="inlineStr"/>
+      <c r="T54" s="7" t="inlineStr">
+        <is>
+          <t>Dépend STK-803</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>STK-805</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Règle métier : refus stock insuffisant</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>Vente REFUSÉE si requested &gt; available — remplace l'écrêtage à 0</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>Cœur du cahier des charges (§3/§18/§19/§20, NON négociable) : avant = vente enregistrée + stock écrêté Math.max(0, …) + note « stock épuisé » (quick-sale.ts:114-123, flag stockShort non bloquant) ; après = refus serveur (autorité) + pré-vérification client pour l'UX → Tata : « Tu as seulement 7 kilos de tomates en stock. Je ne peux pas enregistrer cette vente. » Correction « Alors vends seulement 10 kilos » supportée. Cas exact (=) autorisé, stock 0 → « Tu n'as plus de stock pour ce produit. ». 3 points client alignés (quick-sale, caisse-screen, voice-modal). ⚠ CHANGEMENT DE CONTRAT demandé expressément : le test quick-sale.test.ts « survente signalée sans blocage » est RÉÉCRIT pour acter le refus. Aucune vente, aucun mouvement SALE, aucun stock négatif en cas de refus.</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>STK-804</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>src/lib/quick-sale.ts, src/lib/stock/stock-service.ts, src/components/marchand/caisse-screen.tsx, voice-modal.tsx, vente-rapide-modal.tsx, src/lib/voice/tata-phrases.ts, src/lib/__tests__/quick-sale.test.ts</t>
+        </is>
+      </c>
+      <c r="M55" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N55" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O55" s="4" t="inlineStr"/>
+      <c r="P55" s="4" t="inlineStr">
+        <is>
+          <t>P0 du chantier — la seule modification du flux d'enregistrement existant, demandée par le cahier des charges</t>
+        </is>
+      </c>
+      <c r="Q55" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R55" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S55" s="4" t="inlineStr"/>
+      <c r="T55" s="4" t="inlineStr">
+        <is>
+          <t>Après STK-804 (balance disponible)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>STK-806</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Unités locales CI + conversions</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>kg/sac/carton/bassine/panier/tas… configurables par produit/marchand</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>Aucune supposition universelle sac=X kg : conversion configurable par produit/marchand (merchant_product_units, STK-802). Unité de base par produit (ex. oignons base kg, sac=25 OU 50 kg selon le marchand). Stock réel TOUJOURS en unité de base ; affichage commercial « 2 sacs + 13 kg » (formatStockDisplay). Décimales supportées (numeric(14,3)) pour kg/litre ; entiers pour sac/panier. Seuils low_stock_threshold paramétrables par produit (fini le 10 codé en dur à 5 endroits : stock-store.ts, stock-screen.tsx ×2, caisse-screen.tsx ×2). Avertissement stock faible NON bloquant (§39) — le blocage ne se fait que si requested &gt; available.</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I56" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K56" s="7" t="inlineStr">
+        <is>
+          <t>STK-804</t>
+        </is>
+      </c>
+      <c r="L56" s="7" t="inlineStr">
+        <is>
+          <t>src/lib/stock/units.ts (nouveau), stock-service.ts, stock-store.ts, stock-screen.tsx, caisse-screen.tsx</t>
+        </is>
+      </c>
+      <c r="M56" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N56" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O56" s="7" t="inlineStr"/>
+      <c r="P56" s="7" t="inlineStr">
+        <is>
+          <t>Support profils : le détaillant voit la version simple, grossiste les conversions avancées</t>
+        </is>
+      </c>
+      <c r="Q56" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R56" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S56" s="7" t="inlineStr"/>
+      <c r="T56" s="7" t="inlineStr"/>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>STK-807</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Vocal stock Tata</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>Intents stock_check/loss/adjust/purchase + unités étendues + confirmations</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>localIntent.ts : intents stock_check (« Il reste combien de tomates ? », « Quel est mon stock d'oignons ? » — arbitrage avec navigation 'stock' : présence produit/combien → stock_check), stock_loss (« perdu/gâtées/avariées/cassées/volées »), stock_adjust (« Ajoute 20 kilos », « Enlève 5 kilos », « j'ai compté, il reste 30 kilos »), purchase (« j'ai acheté 2 sacs d'oignons à 12 000 le sac » — discrimine expense par produit du vocabulaire). extractQuantity étendu : bassine/panier/bidon/fût/seau/litre/sachet/régime/plateau/boîte/botte + décimales « 1,5 kilo » + unité remontée dans ParsedIntent. Montant-sans-quantité (« pour 1 500 francs de tomates ») : pendingQuantity → « Tu as vendu combien de kilos de tomates ? » (jamais de décrément arbitraire, §12). Confirmations réutilisant routeConfirmResponse pour opérations ambiguës (§17). Phrases tata-phrases.ts : refus exact, stock faible, consultation convertie (« Il te reste 63 kilos, soit environ 2 sacs et 13 kilos »). Formulations ivoiriennes : 5 mille, un tas, deux paniers, on m'a livré, les tomates sont gâtées…</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>STK-806</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>src/lib/voice/localIntent.ts, tata-phrases.ts, voice-modal.tsx, vente-rapide-modal.tsx + tests __tests__</t>
+        </is>
+      </c>
+      <c r="M57" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N57" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O57" s="4" t="inlineStr"/>
+      <c r="P57" s="4" t="inlineStr">
+        <is>
+          <t>Pipeline vocal inchangé (STT → intent → entités → validation → StockService → RPC → TTS)</t>
+        </is>
+      </c>
+      <c r="Q57" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R57" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S57" s="4" t="inlineStr"/>
+      <c r="T57" s="4" t="inlineStr">
+        <is>
+          <t>Dépend STK-806 (unités)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>STK-808</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Offline/sync stock</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>operation_id + entités queue + conflits métier + refresh balances</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>operation_id UUID généré localement pour toute opération stock (achat, perte, ajustement, transfert) — ventes conservent clientId existant (déjà idempotent). Nouvelles entités de queue + handlers : purchase, stock-movement, stock-transfer (+stock-transfer-receive). Conflit métier : vente offline dont la synchro rencontre INSUFFICIENT_STOCK → 422 → SyncConflictError (mécanisme existant) → conflit rapporté + balance corrigée au refresh. Après chaque flush réussi : rechargement des balances serveur (source de vérité). Vérification locale = pré-vérification UX ; l'autorité reste le serveur (FOR UPDATE + CHECK ≥ 0). Double synchro = 1 seul effet (UNIQUE(merchant_id, operation_id)).</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I58" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K58" s="7" t="inlineStr">
+        <is>
+          <t>STK-804</t>
+        </is>
+      </c>
+      <c r="L58" s="7" t="inlineStr">
+        <is>
+          <t>src/lib/offline-db.ts, src/lib/sync-handlers.ts, src/lib/stock/stock-service.ts, docs/OFFLINE.md</t>
+        </is>
+      </c>
+      <c r="M58" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N58" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O58" s="7" t="inlineStr"/>
+      <c r="P58" s="7" t="inlineStr">
+        <is>
+          <t>Cap file 500 inchangée ; rejeu idempotent garanti serveur</t>
+        </is>
+      </c>
+      <c r="Q58" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R58" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S58" s="7" t="inlineStr"/>
+      <c r="T58" s="7" t="inlineStr"/>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>STK-809</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Transferts, retours, réception, producteur</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>TRANSFER_OUT/IN + retours + commande livrée → stock + PRODUCTION récolte</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Transferts entre marchands (grossiste → semi-grossiste) : merchant_transfer_out (TRANSFER_OUT chez l'expéditeur) + merchant_transfer_receive (TRANSFER_IN chez le destinataire), identifiant commun transfer_id (§28). Retours client (CUSTOMER_RETURN +) et fournisseur (SUPPLIER_RETURN −). Réception d'une commande fournisseur livrée (legacy_supplier_orders status=livree) → achat + mouvement RECEIPT + balance (aujourd'hui la livraison ne réincrémente JAMAIS le stock — gap confirmé). Producteur : « j'ai récolté 100 kilos de tomates » → mouvement PRODUCTION +100 (rôle producteur existant, producteur-store).</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K59" s="4" t="inlineStr">
+        <is>
+          <t>STK-808</t>
+        </is>
+      </c>
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>stock-service.ts, api/marchand/stock/transfers, api/marchand/supplier-orders (réception), producteur-store.ts, api/producteur/*</t>
+        </is>
+      </c>
+      <c r="M59" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N59" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O59" s="4" t="inlineStr"/>
+      <c r="P59" s="4" t="inlineStr">
+        <is>
+          <t>Transferts inter-marchands = 2 transactions liées (pas d'atomicité cross-compte)</t>
+        </is>
+      </c>
+      <c r="Q59" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R59" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S59" s="4" t="inlineStr"/>
+      <c r="T59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>STK-810</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>Prix multi-niveaux + coût moyen + marge</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>PURCHASE/RETAIL/WHOLESALE/SEMI_WHOLESALE + coût moyen pondéré + MARGIN_CHECK</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>merchant_product_prices : prix achat/détail/gros/semi-gros par produit, validité temporelle (§29). Coût moyen pondéré maintenu dans merchant_stock_balances à chaque PURCHASE/ADJUSTMENT_IN (ex. 100 kg × 300 puis 50 kg × 400 → 150 kg à 333,33) (§30). Marge estimée à la vente = (prix vente − coût moyen) × qté, retournée par la RPC. Vocal MARGIN_CHECK (« quelle est ma marge ? ») + PURCHASE_SUMMARY. UI discrète (pas un ERP).</t>
+        </is>
+      </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H60" s="7" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I60" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K60" s="7" t="inlineStr">
+        <is>
+          <t>STK-809</t>
+        </is>
+      </c>
+      <c r="L60" s="7" t="inlineStr">
+        <is>
+          <t>stock-service.ts, api/marchand/stock/prices, localIntent.ts, tata-phrases.ts</t>
+        </is>
+      </c>
+      <c r="M60" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N60" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O60" s="7" t="inlineStr"/>
+      <c r="P60" s="7" t="inlineStr">
+        <is>
+          <t>V1 = coût moyen pondéré uniquement (FIFO/DEPP plus tard)</t>
+        </is>
+      </c>
+      <c r="Q60" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R60" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S60" s="7" t="inlineStr"/>
+      <c r="T60" s="7" t="inlineStr"/>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>STK-811</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>UI stock marchand</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>MES PRODUITS enrichi + historique + perte/comptage — simple, pas un ERP</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>stock-screen.tsx : MES PRODUITS avec stock en unité commerciale (Tomates 18 kg, Oignons 4 sacs + 8 kg, Bananes 3 régimes), badge stock faible basé sur le seuil paramétrable, actions rapides VENDRE / AJOUTER / SIGNALER PERTE / COMPTAGE (ajustement par inventaire §22), historique du produit (18 sept. 09:10 Achat +50 kg… stock actuel 35 kg §43). Variantes par merchantCategorie : détaillant = ultra-simple (Vendre/Ajouter/Voir/Corriger), semi-grossiste/grossiste = + transferts/fournisseurs/prix. Le vocal masque la complexité (§37).</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I61" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>STK-806</t>
+        </is>
+      </c>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
+          <t>src/components/marchand/stock-screen.tsx (+ composants stock/)</t>
+        </is>
+      </c>
+      <c r="M61" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O61" s="4" t="inlineStr"/>
+      <c r="P61" s="4" t="inlineStr">
+        <is>
+          <t>Ne pas transformer Jùlaba en ERP — 5 actions rapides max en surface</t>
+        </is>
+      </c>
+      <c r="Q61" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R61" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S61" s="4" t="inlineStr"/>
+      <c r="T61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>STK-812</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>Tests critiques stock</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>vitest + pgTAP — checklist §46 complète</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>vitest : stock-service (vente ≤ / = / &gt; stock, stock 0, jamais négatif), unités &amp; conversions (kg/sac/carton/bassine/panier par marchand), vocal (phrases ivoiriennes, montant-sans-quantité, refus + correction « alors vends seulement 10 »), offline (achat/perte offline, double synchro = 1 effet, conflit insuffisant), régression ventes/caisse/résumé du jour (694 tests existants restent verts sauf le contrat survente réécrit assumé STK-805). pgTAP : RPC idempotente, CHECK quantity_base ≥ 0, concurrence 2 sessions FOR UPDATE (7+5 sur 10 → une réussit une échoue), RLS default deny, append-only (pas d'UPDATE/DELETE). Definition of Done = checklist §46 du cahier des charges (25 critères).</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I62" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K62" s="7" t="inlineStr">
+        <is>
+          <t>STK-805</t>
+        </is>
+      </c>
+      <c r="L62" s="7" t="inlineStr">
+        <is>
+          <t>src/lib/stock/__tests__/**, src/lib/voice/__tests__/**, supabase/tests/*.sql</t>
+        </is>
+      </c>
+      <c r="M62" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N62" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O62" s="7" t="inlineStr"/>
+      <c r="P62" s="7" t="inlineStr">
+        <is>
+          <t>Transverse — exécuté en continu à chaque STK-8xx</t>
+        </is>
+      </c>
+      <c r="Q62" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R62" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S62" s="7" t="inlineStr"/>
+      <c r="T62" s="7" t="inlineStr"/>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>INF-401</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Déploiement prod + APK</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>Vercel puis APK autonome</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>Déployer prod (Vercel) puis régénérer l'APK SANS CAPACITOR_SERVER_URL (l'APK actuel dépend de la preview sandbox éphémère).</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>ORCHESTRATEUR</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L63" s="4" t="inlineStr">
+        <is>
+          <t>capacitor.config.ts, docs/CAPACITOR.md</t>
+        </is>
+      </c>
+      <c r="M63" s="4" t="inlineStr">
+        <is>
+          <t>Smoke APK</t>
+        </is>
+      </c>
+      <c r="N63" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O63" s="4" t="inlineStr"/>
+      <c r="P63" s="4" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q63" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="R63" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="S63" s="4" t="inlineStr"/>
+      <c r="T63" s="4" t="inlineStr">
+        <is>
+          <t>Rebuild Gradle re-téléchargera les caches purgés (~5 min+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>SEC-402</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>PAT GitHub exposé</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>Révocation</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>PAT ghp_EUGEmf… collé en clair dans les échanges — à révoquer/rotater immédiatement côté compte GitHub.</t>
+        </is>
+      </c>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="H64" s="13" t="inlineStr">
+        <is>
+          <t>BLOQUÉ</t>
+        </is>
+      </c>
+      <c r="I64" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K64" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L64" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M64" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N64" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O64" s="7" t="inlineStr"/>
+      <c r="P64" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q64" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="R64" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="S64" s="7" t="inlineStr"/>
+      <c r="T64" s="7" t="inlineStr">
+        <is>
           <t>Action utilisateur requise — P0 absolu</t>
         </is>
       </c>
     </row>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55">
-      <c r="B55" s="2" t="inlineStr">
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="B56" s="2" t="inlineStr">
+    <row r="68">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>Historique antérieur au 2026-09-18 : voir worklog.md (racine du dépôt, versionné) — Tasks 1-41 (Identificateur, Backoffice, Supabase, voix offline, APK, fix CSP).</t>
         </is>

</xml_diff>

<commit_message>
docs(audit): AUDIT-001 global 77/100 + gouvernance complète + resync registres (Task 67)
- .ai/AUDITS/AUDIT-001-2026-09-19.md : 2 sous-audits (sécurité, cohérence),
  dette, conformité 78 % + preuves live DB (matrice ACL 8/8 RPC merchant_* :
  anon/authenticated/PUBLIC sans EXECUTE, service_role seul ; device_push_tokens
  RLS deny-all) — SEC-813/814 fermées définitivement
- registres créés : AUDIT_REPORT, DEBT_REPORT, SYSTEM_COMPLIANCE, SECURITY_AUDIT,
  SEC_BUGS, TEAM_STATUS, COMMIT_LOG, REVIEW_LOG, LESSONS_LEARNED, INCIDENTS,
  DAILY_STANDUP, ADR-001/002/003 + TEMPLATE, HANDOFF/TEAM_TO_AUDIT
- BUG-002 ouvert (P2) : intent vocal restock = PATCH absolu, contredit D3
- resync : ARCHITECTURE/PROJECT_CONTEXT/OFFLINE (COH-003/004/006/007), TASKS.md
  §8 + ordre d'exécution, TASKS.xlsx (71 tâches, statuts NORM/STK réels),
  CHANGELOG (entrée Task 67, couvre aussi eca2baf/0f71025 — COH-005)
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -124,6 +124,9 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:T68"/>
+  <dimension ref="B2:T79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3056,7 +3059,7 @@
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>TERMINÉ</t>
+          <t>FERMÉ</t>
         </is>
       </c>
       <c r="I32" s="9" t="n">
@@ -3109,12 +3112,12 @@
       </c>
       <c r="S32" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="T32" s="7" t="inlineStr">
         <is>
-          <t>Refs d'indirection + useEffect ; commit b0a95e1</t>
+          <t>b0a95e1</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3154,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I33" s="6" t="n">
@@ -3194,10 +3197,14 @@
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="S33" s="4" t="inlineStr"/>
+      <c r="S33" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>Risque de conflit avec la roadmap — séquencement à arbitrer</t>
+          <t>27ce3da — Task 66 · -867/+511 lignes</t>
         </is>
       </c>
     </row>
@@ -3321,7 +3328,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I35" s="6" t="n">
@@ -3364,8 +3371,16 @@
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="S35" s="4" t="inlineStr"/>
-      <c r="T35" s="4" t="inlineStr"/>
+      <c r="S35" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T35" s="4" t="inlineStr">
+        <is>
+          <t>75a07e1 — Task 66 · CI npm cassée en cascade, réparée par COR-001</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="B36" s="7" t="inlineStr">
@@ -3400,7 +3415,7 @@
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I36" s="9" t="n">
@@ -3443,8 +3458,16 @@
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="S36" s="7" t="inlineStr"/>
-      <c r="T36" s="7" t="inlineStr"/>
+      <c r="S36" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T36" s="7" t="inlineStr">
+        <is>
+          <t>6675cb3 — Task 66 · volet TTS→Zustand ajourné avec justification</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="B37" s="4" t="inlineStr">
@@ -3479,7 +3502,7 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>BLOQUÉ</t>
         </is>
       </c>
       <c r="I37" s="6" t="n">
@@ -3522,8 +3545,16 @@
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="S37" s="4" t="inlineStr"/>
-      <c r="T37" s="4" t="inlineStr"/>
+      <c r="S37" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T37" s="4" t="inlineStr">
+        <is>
+          <t>Docker requis (npx supabase gen types) — procédure documentée dans admin.ts</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="B38" s="7" t="inlineStr">
@@ -4776,7 +4807,7 @@
       </c>
       <c r="H52" s="12" t="inlineStr">
         <is>
-          <t>VALIDATION</t>
+          <t>VALIDATION 90 %</t>
         </is>
       </c>
       <c r="I52" s="9" t="n">
@@ -4823,10 +4854,14 @@
           <t>2026-09-19</t>
         </is>
       </c>
-      <c r="S52" s="7" t="inlineStr"/>
+      <c r="S52" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="T52" s="7" t="inlineStr">
         <is>
-          <t>LIVRÉ Task 62 : 9 tables additives (business_partners, merchant_product_units, merchant_product_prices, merchant_stock_balances CHECK≥0 + stock_precision + low_stock_threshold + weighted_avg_cost, merchant_stock_movements append-only 14 types signés UNIQUE(merchant_id, operation_id) + trigger anti-rewrite, merchant_purchases(+items), merchant_stock_transfers(+items)) + merchant_backfill_opening_balances() idempotent (balance EXACT pour tout produit actif, OPENING_BALANCE si stock&gt;0, operation_id déterministe md5) · application en base : bun run supabase:push au moment de la bascule STK-804/805</t>
+          <t>Fondation SQL appliquée en prod + pgTAP 108</t>
         </is>
       </c>
     </row>
@@ -4863,7 +4898,7 @@
       </c>
       <c r="H53" s="11" t="inlineStr">
         <is>
-          <t>VALIDATION</t>
+          <t>VALIDATION 90 %</t>
         </is>
       </c>
       <c r="I53" s="6" t="n">
@@ -4910,10 +4945,14 @@
           <t>2026-09-19</t>
         </is>
       </c>
-      <c r="S53" s="4" t="inlineStr"/>
+      <c r="S53" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="T53" s="4" t="inlineStr">
         <is>
-          <t>LIVRÉ Task 62 : merchant_record_sale (FOR UPDATE tri product_id anti-deadlock, refus strict, contrat vente actuel préservé : total recalculé serveur + change écrêté + idempotence client_id = operation_id, double écriture D3, produit sans balance/UNKNOWN → vente encaissée sans mouvement) · merchant_record_purchase (PURCHASE + coût moyen pondéré + balance créée EXACT au 1er achat + dépense liée optionnelle D6) · merchant_record_movement (entrées créent la balance, sorties UNKNOWN → UNKNOWN_STOCK, reason obligatoire, SALE/PURCHASE/TRANSFER_*/OPENING_BALANCE redirigés) · merchant_adjust_to_count (delta tracé, comptage UNKNOWN → before=0, balance passée EXACT) · security definer, revoke public, grant service_role uniquement · transferts STK-809</t>
+          <t>RPC appliquées en prod (fixes 110000/110100)</t>
         </is>
       </c>
     </row>
@@ -4950,7 +4989,7 @@
       </c>
       <c r="H54" s="12" t="inlineStr">
         <is>
-          <t>VALIDATION</t>
+          <t>VALIDATION 90 %</t>
         </is>
       </c>
       <c r="I54" s="9" t="n">
@@ -4997,10 +5036,14 @@
           <t>2026-09-19</t>
         </is>
       </c>
-      <c r="S54" s="7" t="inlineStr"/>
+      <c r="S54" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="T54" s="7" t="inlineStr">
         <is>
-          <t>LIVRÉ Task 62 : bascule ventes sur RPC transactionnelle avec refus strict serveur actif dès le db push · dépend STK-803 (livré)</t>
+          <t>Bascule ventes effective (RPC vivant en prod)</t>
         </is>
       </c>
     </row>
@@ -5037,7 +5080,7 @@
       </c>
       <c r="H55" s="11" t="inlineStr">
         <is>
-          <t>VALIDATION</t>
+          <t>VALIDATION 90 %</t>
         </is>
       </c>
       <c r="I55" s="6" t="n">
@@ -5084,10 +5127,14 @@
           <t>2026-09-19</t>
         </is>
       </c>
-      <c r="S55" s="4" t="inlineStr"/>
+      <c r="S55" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="T55" s="4" t="inlineStr">
         <is>
-          <t>Après STK-804 (livré)</t>
+          <t>Refus strict actif 3 niveaux</t>
         </is>
       </c>
     </row>
@@ -5124,7 +5171,7 @@
       </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>A_FAIRE</t>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I56" s="9" t="n">
@@ -5171,8 +5218,16 @@
           <t>2026-09-19</t>
         </is>
       </c>
-      <c r="S56" s="7" t="inlineStr"/>
-      <c r="T56" s="7" t="inlineStr"/>
+      <c r="S56" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T56" s="7" t="inlineStr">
+        <is>
+          <t>8d9898a — Task 64</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="22" customHeight="1">
       <c r="B57" s="4" t="inlineStr">
@@ -5207,7 +5262,7 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>A_FAIRE</t>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I57" s="6" t="n">
@@ -5254,10 +5309,14 @@
           <t>2026-09-19</t>
         </is>
       </c>
-      <c r="S57" s="4" t="inlineStr"/>
+      <c r="S57" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="T57" s="4" t="inlineStr">
         <is>
-          <t>Dépend STK-806 (unités)</t>
+          <t>2f6367a — Task 64</t>
         </is>
       </c>
     </row>
@@ -5294,7 +5353,7 @@
       </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>A_FAIRE</t>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I58" s="9" t="n">
@@ -5341,8 +5400,16 @@
           <t>2026-09-19</t>
         </is>
       </c>
-      <c r="S58" s="7" t="inlineStr"/>
-      <c r="T58" s="7" t="inlineStr"/>
+      <c r="S58" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T58" s="7" t="inlineStr">
+        <is>
+          <t>ea96e6a — Task 64</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="22" customHeight="1">
       <c r="B59" s="4" t="inlineStr">
@@ -5377,7 +5444,7 @@
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>A_FAIRE</t>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I59" s="6" t="n">
@@ -5424,8 +5491,16 @@
           <t>2026-09-19</t>
         </is>
       </c>
-      <c r="S59" s="4" t="inlineStr"/>
-      <c r="T59" s="4" t="inlineStr"/>
+      <c r="S59" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T59" s="4" t="inlineStr">
+        <is>
+          <t>29333f7 + UI bea5f16 (STK-815) — Tasks 64/66</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="22" customHeight="1">
       <c r="B60" s="7" t="inlineStr">
@@ -5460,7 +5535,7 @@
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>A_FAIRE</t>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I60" s="9" t="n">
@@ -5507,8 +5582,16 @@
           <t>2026-09-19</t>
         </is>
       </c>
-      <c r="S60" s="7" t="inlineStr"/>
-      <c r="T60" s="7" t="inlineStr"/>
+      <c r="S60" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T60" s="7" t="inlineStr">
+        <is>
+          <t>f801dcf — Task 64</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="22" customHeight="1">
       <c r="B61" s="4" t="inlineStr">
@@ -5543,7 +5626,7 @@
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>A_FAIRE</t>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I61" s="6" t="n">
@@ -5590,8 +5673,16 @@
           <t>2026-09-19</t>
         </is>
       </c>
-      <c r="S61" s="4" t="inlineStr"/>
-      <c r="T61" s="4" t="inlineStr"/>
+      <c r="S61" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T61" s="4" t="inlineStr">
+        <is>
+          <t>0f1faac — Task 64</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="22" customHeight="1">
       <c r="B62" s="7" t="inlineStr">
@@ -5626,7 +5717,7 @@
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>A_FAIRE</t>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="I62" s="9" t="n">
@@ -5673,8 +5764,16 @@
           <t>2026-09-19</t>
         </is>
       </c>
-      <c r="S62" s="7" t="inlineStr"/>
-      <c r="T62" s="7" t="inlineStr"/>
+      <c r="S62" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T62" s="7" t="inlineStr">
+        <is>
+          <t>b660e9a — Task 64 · pgTAP 108 · checklist 25/25</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="22" customHeight="1">
       <c r="B63" s="4" t="inlineStr">
@@ -5853,18 +5952,883 @@
     <row r="65"/>
     <row r="66"/>
     <row r="67">
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="B68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>STK-815</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>UI transferts inter-marchands</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Écran + annuaire + fixes contrat</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>transferts-screen.tsx : onglets À recevoir/Envoyés, création multi-lignes (unités honnêtes + équivalent base), offline stock-transfer/stock-transfer-action, refus parlé jamais en file ; route transfers/merchants (annuaire) ; codes TRANSFER_* → 400 + label FR ; GET corrigé (receivedQuantityBase, cancelReason)</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I69" s="14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J69" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K69" s="7" t="inlineStr">
+        <is>
+          <t>STK-809</t>
+        </is>
+      </c>
+      <c r="L69" s="7" t="inlineStr">
+        <is>
+          <t>src/components/marchand/transferts-screen.tsx ; src/app/api/marchand/stock/transfers/* ; src/lib/stock/transfer-ui.ts</t>
+        </is>
+      </c>
+      <c r="M69" s="7" t="inlineStr">
+        <is>
+          <t>transfer-ui.test 16 ; stock-service +1 ; transverse garde littéral</t>
+        </is>
+      </c>
+      <c r="N69" s="7" t="inlineStr">
+        <is>
+          <t>879/879 · tsc 0 · lint 0 · build OK</t>
+        </is>
+      </c>
+      <c r="O69" s="7" t="inlineStr"/>
+      <c r="P69" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q69" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R69" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S69" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T69" s="7" t="inlineStr">
+        <is>
+          <t>bea5f16 — Task 66</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>SEC-813</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>Exposition RPC merchant_* à anon</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>REVOKE EXECUTE anon+authenticated (8 RPC)</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>5 RPC de la migration 20260919100000 + auto-revoke des 3 transfer_* (110200:159/110300:147/110400:96) + ré-appliqué par fixes 110000/110100. VALIDÉ LIVE 2026-09-19 : has_function_privilege anon/authenticated/PUBLIC=false ×8, service_role=true ×8</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>DEV SECURITE</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>FERMÉ</t>
+        </is>
+      </c>
+      <c r="I70" s="14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J70" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K70" s="7" t="inlineStr">
+        <is>
+          <t>STK-803</t>
+        </is>
+      </c>
+      <c r="L70" s="7" t="inlineStr">
+        <is>
+          <t>supabase/migrations/20260919100000*.sql ; scripts/db_acl_check.js, db_svc_check.js (workspace)</t>
+        </is>
+      </c>
+      <c r="M70" s="7" t="inlineStr">
+        <is>
+          <t>pgTAP ACL (stock.sql) ; vérification live re-jouable</t>
+        </is>
+      </c>
+      <c r="N70" s="7" t="inlineStr">
+        <is>
+          <t>108 pgTAP ; preuve live AUDIT-001</t>
+        </is>
+      </c>
+      <c r="O70" s="7" t="inlineStr"/>
+      <c r="P70" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q70" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R70" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S70" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T70" s="7" t="inlineStr">
+        <is>
+          <t>55bbed2 — Task 64 ; matrice dans .ai/SECURITY_AUDIT.md §3</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>SEC-814</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>device_push_tokens exposé (RLS off + anon grants)</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>RLS on + revoke anon/authenticated</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>20260919100100 : RLS activé (0 policy = deny-all), revoke anon+authenticated (TRUNCATE compris). VALIDÉ LIVE 2026-09-19 : grants tables = postgres + service_role uniquement ; route push-tokens dérive le subject du cookie serveur</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>DEV SECURITE</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>FERMÉ</t>
+        </is>
+      </c>
+      <c r="I71" s="14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J71" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K71" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L71" s="7" t="inlineStr">
+        <is>
+          <t>supabase/migrations/20260919100100*.sql ; src/app/api/push-tokens/route.ts</t>
+        </is>
+      </c>
+      <c r="M71" s="7" t="inlineStr">
+        <is>
+          <t>pgTAP ACL ; vérification live</t>
+        </is>
+      </c>
+      <c r="N71" s="7" t="inlineStr">
+        <is>
+          <t>preuve live AUDIT-001</t>
+        </is>
+      </c>
+      <c r="O71" s="7" t="inlineStr"/>
+      <c r="P71" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q71" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R71" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S71" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T71" s="7" t="inlineStr">
+        <is>
+          <t>55bbed2 — Task 64</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>AUDIT-001</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>Audit global</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Audit global périodique #001</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>Cohérence + dette + conformité + santé multi-agents</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>2 sous-audits (sécurité, cohérence) + mesure dette + preuves live DB. Score global 77/100 (sécurité 90, archi 85, tests 85, doc 68 remédiée, perf 65, a11y 55). 0 mensonge détecté, 0 test orphelin</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>AGENT AUDIT</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I72" s="14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J72" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K72" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L72" s="7" t="inlineStr">
+        <is>
+          <t>.ai/AUDITS/AUDIT-001-2026-09-19.md ; .ai/AUDIT_REPORT.md</t>
+        </is>
+      </c>
+      <c r="M72" s="7" t="inlineStr">
+        <is>
+          <t>baseline complète : 879/879 · tsc 0 · eslint 0 · build OK</t>
+        </is>
+      </c>
+      <c r="N72" s="7" t="inlineStr">
+        <is>
+          <t>879/879 (55 fichiers)</t>
+        </is>
+      </c>
+      <c r="O72" s="7" t="inlineStr">
+        <is>
+          <t>COH-001→COR-001 ; COH-002→BUG-002</t>
+        </is>
+      </c>
+      <c r="P72" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q72" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R72" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S72" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T72" s="7" t="inlineStr">
+        <is>
+          <t>Task 67 — prochain audit : +5 features ou 2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>COR-001</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Audit global</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>CI GitHub réparée (COH-001)</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>Workflow npm → Bun</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>npm ci + cache npm cassés depuis NORM-303 (package-lock sorti du dépôt) : bascule oven-sh/setup-bun@v2 + bun install --frozen-lockfile + bun run lint/typecheck/test — alignée sur le runtime officiel</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>DEVOPS</t>
+        </is>
+      </c>
+      <c r="H73" s="7" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I73" s="14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J73" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K73" s="7" t="inlineStr">
+        <is>
+          <t>NORM-303</t>
+        </is>
+      </c>
+      <c r="L73" s="7" t="inlineStr">
+        <is>
+          <t>.github/workflows/ci.yml</t>
+        </is>
+      </c>
+      <c r="M73" s="7" t="inlineStr">
+        <is>
+          <t>run CI à vérifier au premier push (action GitHub)</t>
+        </is>
+      </c>
+      <c r="N73" s="7" t="inlineStr">
+        <is>
+          <t>à confirmer sur GitHub Actions</t>
+        </is>
+      </c>
+      <c r="O73" s="7" t="inlineStr"/>
+      <c r="P73" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q73" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R73" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S73" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T73" s="7" t="inlineStr">
+        <is>
+          <t>Task 67 · leçon L-004/L-006</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>DOC-307</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>Audit global</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>Resync docs de pilotage (COH-003/004)</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>ARCHITECTURE.md + PROJECT_CONTEXT.md</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>Métriques resynchronisées : 85 routes, 136 migrations, ~99 tables, 91 050 l., localIntent 905 l. + voice-stock, 18 handlers, baseline 879/879 ; doublons §6 résolus marqués (NORM-301/303/304) ; NORM-304 « ajourné avec justification »</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>AGENT 2</t>
+        </is>
+      </c>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I74" s="14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J74" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K74" s="7" t="inlineStr">
+        <is>
+          <t>AUDIT-001</t>
+        </is>
+      </c>
+      <c r="L74" s="7" t="inlineStr">
+        <is>
+          <t>.ai/ARCHITECTURE.md ; .ai/PROJECT_CONTEXT.md</t>
+        </is>
+      </c>
+      <c r="M74" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N74" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O74" s="7" t="inlineStr"/>
+      <c r="P74" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q74" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R74" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S74" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T74" s="7" t="inlineStr">
+        <is>
+          <t>Task 67</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>DOC-308</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Audit global</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>Resync docs/OFFLINE.md (COH-006)</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>Matrice marchand + scénario réappro</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>Réappro absolu retiré de la matrice (supprimé STK-811) ; réappro/perte/comptage via actions stock delta + operation_id ; entités stock offline documentées (stock-movement/count/purchase/transfer/transfer-action/reception)</t>
+        </is>
+      </c>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>AGENT 2</t>
+        </is>
+      </c>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I75" s="14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J75" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="K75" s="7" t="inlineStr">
+        <is>
+          <t>AUDIT-001</t>
+        </is>
+      </c>
+      <c r="L75" s="7" t="inlineStr">
+        <is>
+          <t>docs/OFFLINE.md</t>
+        </is>
+      </c>
+      <c r="M75" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N75" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O75" s="7" t="inlineStr"/>
+      <c r="P75" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q75" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R75" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S75" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T75" s="7" t="inlineStr">
+        <is>
+          <t>Task 67</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>GOV-309</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>Audit global</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Registres de gouvernance créés</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>Initialisation registres manquants</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>AUDIT_REPORT, DEBT_REPORT (8 items, 0 critique), SYSTEM_COMPLIANCE (78 %), SECURITY_AUDIT (+ matrice live), SEC_BUGS (SEC-OBS-2/3/4), TEAM_STATUS, COMMIT_LOG, REVIEW_LOG, LESSONS_LEARNED (8 leçons), INCIDENTS (3), DAILY_STANDUP, ADR-001/002/003 + TEMPLATE, HANDOFF/TEAM_TO_AUDIT</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>AGENT AUDIT</t>
+        </is>
+      </c>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I76" s="14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J76" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K76" s="7" t="inlineStr">
+        <is>
+          <t>AUDIT-001</t>
+        </is>
+      </c>
+      <c r="L76" s="7" t="inlineStr">
+        <is>
+          <t>.ai/* (19 fichiers)</t>
+        </is>
+      </c>
+      <c r="M76" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N76" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O76" s="7" t="inlineStr"/>
+      <c r="P76" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="Q76" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R76" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S76" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="T76" s="7" t="inlineStr">
+        <is>
+          <t>Task 67</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>BUG-002</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Correction</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Intent vocal restock = PATCH absolu (COH-002)</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>Router sur merchant_record_purchase</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>voice-modal.tsx:245 fait updateProduct(stockQty+qty) via file product-update : contredit D3/STK-805/STK-811 (dérive balance↔stock_qty, aucun mouvement PURCHASE). Correctif : RPC achat + delta local adjustLocalStock + file stock-purchase + refus parlé. Spec courte + tests AVANT code</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>AGENT 1</t>
+        </is>
+      </c>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>OUVERT</t>
+        </is>
+      </c>
+      <c r="I77" s="14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J77" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K77" s="7" t="inlineStr">
+        <is>
+          <t>STK-807</t>
+        </is>
+      </c>
+      <c r="L77" s="7" t="inlineStr">
+        <is>
+          <t>src/components/marchand/voice-modal.tsx ; src/lib/stores/stock-store.ts</t>
+        </is>
+      </c>
+      <c r="M77" s="7" t="inlineStr">
+        <is>
+          <t>test dédié intent restock → achat RPC (à écrire)</t>
+        </is>
+      </c>
+      <c r="N77" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O77" s="7" t="inlineStr">
+        <is>
+          <t>BUG-002</t>
+        </is>
+      </c>
+      <c r="P77" s="7" t="inlineStr">
+        <is>
+          <t>Dérive silencieuse des stocks</t>
+        </is>
+      </c>
+      <c r="Q77" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="R77" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="S77" s="7" t="inlineStr"/>
+      <c r="T77" s="7" t="inlineStr">
+        <is>
+          <t>Détecté AUDIT-001 · prochain chantier</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Historique antérieur au 2026-09-18 : voir worklog.md (racine du dépôt, versionné) — Tasks 1-41 (Identificateur, Backoffice, Supabase, voix offline, APK, fix CSP).</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="7" t="inlineStr">
         <is>
           <t>Notes : la Progression reflète l'état RÉEL (règle 16 du protocole) — une tâche n'est jamais 100 % sans test + validation AGENT 2. Le registre TASKS.xlsx prime sur TASKS.md (miroir).</t>
         </is>
       </c>
-    </row>
-    <row r="68">
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Historique antérieur au 2026-09-18 : voir worklog.md (racine du dépôt, versionné) — Tasks 1-41 (Identificateur, Backoffice, Supabase, voix offline, APK, fix CSP).</t>
-        </is>
-      </c>
+      <c r="C79" s="7" t="n"/>
+      <c r="D79" s="7" t="n"/>
+      <c r="E79" s="7" t="n"/>
+      <c r="F79" s="7" t="n"/>
+      <c r="G79" s="7" t="n"/>
+      <c r="H79" s="7" t="n"/>
+      <c r="I79" s="14" t="n"/>
+      <c r="J79" s="7" t="n"/>
+      <c r="K79" s="7" t="n"/>
+      <c r="L79" s="7" t="n"/>
+      <c r="M79" s="7" t="n"/>
+      <c r="N79" s="7" t="n"/>
+      <c r="O79" s="7" t="n"/>
+      <c r="P79" s="7" t="n"/>
+      <c r="Q79" s="7" t="n"/>
+      <c r="R79" s="7" t="n"/>
+      <c r="S79" s="7" t="n"/>
+      <c r="T79" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>